<commit_message>
WIP: cambios locales pendientes de subir
Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/BD_Maquinaria_y_Partes.xlsx
+++ b/BD_Maquinaria_y_Partes.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fjha_\Downloads\GESTION 3.0\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F3FB5DB1-2C95-4B90-86BF-F0569B4F8782}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B8A9407B-21BA-42C9-BFC7-FAB89BA72B5B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="30936" windowHeight="16776" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -22,7 +22,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="875" uniqueCount="448">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1210" uniqueCount="517">
   <si>
     <t>BASE DE DATOS — MAQUINARIA</t>
   </si>
@@ -1260,12 +1260,6 @@
     <t>DETECTORES</t>
   </si>
   <si>
-    <t>EQUIPOS</t>
-  </si>
-  <si>
-    <t>COMPRESORES</t>
-  </si>
-  <si>
     <t>ELECTRICO</t>
   </si>
   <si>
@@ -1296,9 +1290,6 @@
     <t>PUERTAS</t>
   </si>
   <si>
-    <t>COMPRESOR</t>
-  </si>
-  <si>
     <t>CARRO</t>
   </si>
   <si>
@@ -1366,6 +1357,222 @@
   </si>
   <si>
     <t>B</t>
+  </si>
+  <si>
+    <t>FRIO EQUIPO1</t>
+  </si>
+  <si>
+    <t>FRIO EQUIPOS</t>
+  </si>
+  <si>
+    <t>FRIO COMPRESORES</t>
+  </si>
+  <si>
+    <t>FRIO EQUIPO2</t>
+  </si>
+  <si>
+    <t>FRIO COMPRESOR</t>
+  </si>
+  <si>
+    <t>FRIO COMPRESOR 1</t>
+  </si>
+  <si>
+    <t>FRIO COMPRESOR 2</t>
+  </si>
+  <si>
+    <t>FRIO EQUIPO 1</t>
+  </si>
+  <si>
+    <t>FRIO EQUIPO 2</t>
+  </si>
+  <si>
+    <t>FRIO EQUIPO 3</t>
+  </si>
+  <si>
+    <t>FRIO EQUIPO 4</t>
+  </si>
+  <si>
+    <t>FRIO COMPRESOR 3</t>
+  </si>
+  <si>
+    <t>FRIO COMPRESOR 4</t>
+  </si>
+  <si>
+    <t>CAMARA STOCK 1</t>
+  </si>
+  <si>
+    <t>CAMARA STOCK 2</t>
+  </si>
+  <si>
+    <t>CAMARA STOCK 3</t>
+  </si>
+  <si>
+    <t>CAMARA STOCK 4</t>
+  </si>
+  <si>
+    <t>CAMARA STOCK 5 (TRUENO)</t>
+  </si>
+  <si>
+    <t>TANQUE 1</t>
+  </si>
+  <si>
+    <t>TANQUE 2</t>
+  </si>
+  <si>
+    <t>TANQUE 3</t>
+  </si>
+  <si>
+    <t>TANQUE 4</t>
+  </si>
+  <si>
+    <t>TANQUE 5 (TRUENO)</t>
+  </si>
+  <si>
+    <t>A/A OBRADOR</t>
+  </si>
+  <si>
+    <t>A/A VESTUARIO</t>
+  </si>
+  <si>
+    <t>A/A OFICINAS</t>
+  </si>
+  <si>
+    <t>A/A</t>
+  </si>
+  <si>
+    <t>FRIO EQUIPO</t>
+  </si>
+  <si>
+    <t>AGUA</t>
+  </si>
+  <si>
+    <t>BOYA</t>
+  </si>
+  <si>
+    <t>NIVEL</t>
+  </si>
+  <si>
+    <t>BOMBAS</t>
+  </si>
+  <si>
+    <t>SERVO</t>
+  </si>
+  <si>
+    <t>ZELAIETA</t>
+  </si>
+  <si>
+    <t>BPF</t>
+  </si>
+  <si>
+    <t>INFRIMA</t>
+  </si>
+  <si>
+    <t>CONDENSADORES ELECTRICOS</t>
+  </si>
+  <si>
+    <t>CUADROS GENERALES</t>
+  </si>
+  <si>
+    <t>MAQ-148</t>
+  </si>
+  <si>
+    <t>MAQ-149</t>
+  </si>
+  <si>
+    <t>MAQ-150</t>
+  </si>
+  <si>
+    <t>MAQ-151</t>
+  </si>
+  <si>
+    <t>MAQ-152</t>
+  </si>
+  <si>
+    <t>MAQ-153</t>
+  </si>
+  <si>
+    <t>MAQ-154</t>
+  </si>
+  <si>
+    <t>MAQ-155</t>
+  </si>
+  <si>
+    <t>MAQ-156</t>
+  </si>
+  <si>
+    <t>MAQ-157</t>
+  </si>
+  <si>
+    <t>MAQ-158</t>
+  </si>
+  <si>
+    <t>MAQ-159</t>
+  </si>
+  <si>
+    <t>MAQ-160</t>
+  </si>
+  <si>
+    <t>MAQ-161</t>
+  </si>
+  <si>
+    <t>MAQ-162</t>
+  </si>
+  <si>
+    <t>MAQ-163</t>
+  </si>
+  <si>
+    <t>MAQ-164</t>
+  </si>
+  <si>
+    <t>MAQ-165</t>
+  </si>
+  <si>
+    <t>MAQ-166</t>
+  </si>
+  <si>
+    <t>MAQ-167</t>
+  </si>
+  <si>
+    <t>MAQ-168</t>
+  </si>
+  <si>
+    <t>MAQ-169</t>
+  </si>
+  <si>
+    <t>MAQ-170</t>
+  </si>
+  <si>
+    <t>ELECTRICIDAD</t>
+  </si>
+  <si>
+    <t>JACGA</t>
+  </si>
+  <si>
+    <t>NAVES</t>
+  </si>
+  <si>
+    <t>A/A MUELLE</t>
+  </si>
+  <si>
+    <t>EXTRACTORES RELAMPAGO</t>
+  </si>
+  <si>
+    <t>EXTRACTORES TRUENO</t>
+  </si>
+  <si>
+    <t>EVAPORATIVAS</t>
+  </si>
+  <si>
+    <t>EXTRACTORES</t>
+  </si>
+  <si>
+    <t>CANALIZACION</t>
+  </si>
+  <si>
+    <t>FILTROS</t>
+  </si>
+  <si>
+    <t>OTROS</t>
   </si>
 </sst>
 </file>
@@ -1570,7 +1777,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -1599,6 +1806,21 @@
     <xf numFmtId="0" fontId="7" fillId="7" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="7" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
@@ -1620,23 +1842,6 @@
     </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="7" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="11" borderId="0" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="11" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1965,7 +2170,7 @@
   <sheetPr>
     <tabColor rgb="FF1F4E79"/>
   </sheetPr>
-  <dimension ref="A1:R150"/>
+  <dimension ref="A1:R173"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="13" customWidth="1"/>
@@ -1979,32 +2184,32 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:18" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="13" t="s">
+      <c r="A1" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="19"/>
     </row>
     <row r="2" spans="1:18" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="15" t="s">
+      <c r="A2" s="20" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-      <c r="I2" s="14"/>
-      <c r="J2" s="14"/>
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+      <c r="I2" s="19"/>
+      <c r="J2" s="19"/>
     </row>
     <row r="3" spans="1:18" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
@@ -2063,15 +2268,15 @@
       <c r="J4" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="L4" s="16"/>
-      <c r="M4" s="16"/>
-      <c r="N4" s="12" t="s">
+      <c r="L4" s="21"/>
+      <c r="M4" s="21"/>
+      <c r="N4" s="17" t="s">
         <v>91</v>
       </c>
-      <c r="O4" s="12"/>
-      <c r="P4" s="12"/>
-      <c r="Q4" s="12"/>
-      <c r="R4" s="12"/>
+      <c r="O4" s="17"/>
+      <c r="P4" s="17"/>
+      <c r="Q4" s="17"/>
+      <c r="R4" s="17"/>
     </row>
     <row r="5" spans="1:18" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="3" t="s">
@@ -2098,15 +2303,15 @@
       <c r="J5" s="4" t="s">
         <v>14</v>
       </c>
-      <c r="L5" s="17"/>
-      <c r="M5" s="17"/>
-      <c r="N5" s="12" t="s">
+      <c r="L5" s="22"/>
+      <c r="M5" s="22"/>
+      <c r="N5" s="17" t="s">
         <v>90</v>
       </c>
-      <c r="O5" s="12"/>
-      <c r="P5" s="12"/>
-      <c r="Q5" s="12"/>
-      <c r="R5" s="12"/>
+      <c r="O5" s="17"/>
+      <c r="P5" s="17"/>
+      <c r="Q5" s="17"/>
+      <c r="R5" s="17"/>
     </row>
     <row r="6" spans="1:18" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A6" s="3" t="s">
@@ -2133,15 +2338,15 @@
       <c r="J6" s="3" t="s">
         <v>14</v>
       </c>
-      <c r="L6" s="18"/>
-      <c r="M6" s="18"/>
-      <c r="N6" s="12" t="s">
+      <c r="L6" s="23"/>
+      <c r="M6" s="23"/>
+      <c r="N6" s="17" t="s">
         <v>89</v>
       </c>
-      <c r="O6" s="12"/>
-      <c r="P6" s="12"/>
-      <c r="Q6" s="12"/>
-      <c r="R6" s="12"/>
+      <c r="O6" s="17"/>
+      <c r="P6" s="17"/>
+      <c r="Q6" s="17"/>
+      <c r="R6" s="17"/>
     </row>
     <row r="7" spans="1:18" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
@@ -2312,7 +2517,7 @@
       </c>
       <c r="I13" s="5"/>
       <c r="J13" s="5" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
     </row>
     <row r="14" spans="1:18" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -2336,7 +2541,7 @@
       </c>
       <c r="I14" s="5"/>
       <c r="J14" s="5" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
     </row>
     <row r="15" spans="1:18" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -2360,7 +2565,7 @@
       </c>
       <c r="I15" s="5"/>
       <c r="J15" s="5" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
     </row>
     <row r="16" spans="1:18" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -2384,7 +2589,7 @@
       </c>
       <c r="I16" s="5"/>
       <c r="J16" s="5" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
     </row>
     <row r="17" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -2408,7 +2613,7 @@
       </c>
       <c r="I17" s="5"/>
       <c r="J17" s="5" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
     </row>
     <row r="18" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -2432,7 +2637,7 @@
       </c>
       <c r="I18" s="5"/>
       <c r="J18" s="5" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
     </row>
     <row r="19" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
@@ -2479,7 +2684,9 @@
         <v>98</v>
       </c>
       <c r="I20" s="5"/>
-      <c r="J20" s="5"/>
+      <c r="J20" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="21" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A21" s="3" t="s">
@@ -2501,7 +2708,9 @@
         <v>98</v>
       </c>
       <c r="I21" s="5"/>
-      <c r="J21" s="5"/>
+      <c r="J21" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="22" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="3" t="s">
@@ -2523,7 +2732,9 @@
         <v>98</v>
       </c>
       <c r="I22" s="5"/>
-      <c r="J22" s="5"/>
+      <c r="J22" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="23" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A23" s="3" t="s">
@@ -2545,7 +2756,9 @@
         <v>98</v>
       </c>
       <c r="I23" s="5"/>
-      <c r="J23" s="5"/>
+      <c r="J23" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="24" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="3" t="s">
@@ -2567,7 +2780,9 @@
         <v>98</v>
       </c>
       <c r="I24" s="5"/>
-      <c r="J24" s="5"/>
+      <c r="J24" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="25" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A25" s="3" t="s">
@@ -2589,7 +2804,9 @@
         <v>98</v>
       </c>
       <c r="I25" s="5"/>
-      <c r="J25" s="5"/>
+      <c r="J25" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="26" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="3" t="s">
@@ -2609,7 +2826,9 @@
         <v>98</v>
       </c>
       <c r="I26" s="5"/>
-      <c r="J26" s="5"/>
+      <c r="J26" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="27" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A27" s="3" t="s">
@@ -2629,7 +2848,9 @@
         <v>98</v>
       </c>
       <c r="I27" s="5"/>
-      <c r="J27" s="5"/>
+      <c r="J27" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="28" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="3" t="s">
@@ -2649,7 +2870,9 @@
         <v>98</v>
       </c>
       <c r="I28" s="5"/>
-      <c r="J28" s="5"/>
+      <c r="J28" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="29" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="3" t="s">
@@ -2669,7 +2892,9 @@
         <v>98</v>
       </c>
       <c r="I29" s="5"/>
-      <c r="J29" s="5"/>
+      <c r="J29" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="30" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="3" t="s">
@@ -2689,7 +2914,9 @@
         <v>98</v>
       </c>
       <c r="I30" s="5"/>
-      <c r="J30" s="5"/>
+      <c r="J30" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="31" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A31" s="3" t="s">
@@ -2709,7 +2936,9 @@
         <v>98</v>
       </c>
       <c r="I31" s="5"/>
-      <c r="J31" s="5"/>
+      <c r="J31" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="32" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="3" t="s">
@@ -2729,7 +2958,9 @@
         <v>98</v>
       </c>
       <c r="I32" s="5"/>
-      <c r="J32" s="5"/>
+      <c r="J32" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="33" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A33" s="3" t="s">
@@ -2749,7 +2980,9 @@
         <v>98</v>
       </c>
       <c r="I33" s="5"/>
-      <c r="J33" s="5"/>
+      <c r="J33" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="34" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="3" t="s">
@@ -2769,7 +3002,9 @@
         <v>98</v>
       </c>
       <c r="I34" s="5"/>
-      <c r="J34" s="5"/>
+      <c r="J34" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="35" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A35" s="3" t="s">
@@ -2789,7 +3024,9 @@
         <v>98</v>
       </c>
       <c r="I35" s="5"/>
-      <c r="J35" s="5"/>
+      <c r="J35" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="36" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="3" t="s">
@@ -2811,7 +3048,9 @@
         <v>98</v>
       </c>
       <c r="I36" s="5"/>
-      <c r="J36" s="5"/>
+      <c r="J36" s="5" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="37" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A37" s="3" t="s">
@@ -2835,7 +3074,9 @@
       <c r="I37" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="J37" s="5"/>
+      <c r="J37" s="5" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="38" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="3" t="s">
@@ -2857,7 +3098,9 @@
         <v>98</v>
       </c>
       <c r="I38" s="5"/>
-      <c r="J38" s="5"/>
+      <c r="J38" s="5" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="39" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A39" s="3" t="s">
@@ -2879,7 +3122,9 @@
         <v>98</v>
       </c>
       <c r="I39" s="5"/>
-      <c r="J39" s="5"/>
+      <c r="J39" s="5" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="40" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="3" t="s">
@@ -2901,7 +3146,9 @@
         <v>98</v>
       </c>
       <c r="I40" s="5"/>
-      <c r="J40" s="5"/>
+      <c r="J40" s="5" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="41" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A41" s="3" t="s">
@@ -2923,7 +3170,9 @@
         <v>98</v>
       </c>
       <c r="I41" s="5"/>
-      <c r="J41" s="5"/>
+      <c r="J41" s="5" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="42" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="3" t="s">
@@ -2945,7 +3194,9 @@
         <v>98</v>
       </c>
       <c r="I42" s="5"/>
-      <c r="J42" s="5"/>
+      <c r="J42" s="5" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="43" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A43" s="3" t="s">
@@ -2967,7 +3218,9 @@
         <v>98</v>
       </c>
       <c r="I43" s="5"/>
-      <c r="J43" s="5"/>
+      <c r="J43" s="5" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="44" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="3" t="s">
@@ -2989,7 +3242,9 @@
         <v>98</v>
       </c>
       <c r="I44" s="5"/>
-      <c r="J44" s="5"/>
+      <c r="J44" s="5" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="45" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A45" s="3" t="s">
@@ -3001,7 +3256,9 @@
       <c r="C45" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="D45" s="5"/>
+      <c r="D45" s="5" t="s">
+        <v>478</v>
+      </c>
       <c r="E45" s="5"/>
       <c r="F45" s="5"/>
       <c r="G45" s="5"/>
@@ -3009,7 +3266,9 @@
         <v>98</v>
       </c>
       <c r="I45" s="5"/>
-      <c r="J45" s="5"/>
+      <c r="J45" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="46" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="3" t="s">
@@ -3021,7 +3280,9 @@
       <c r="C46" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="D46" s="5"/>
+      <c r="D46" s="5" t="s">
+        <v>478</v>
+      </c>
       <c r="E46" s="5"/>
       <c r="F46" s="5"/>
       <c r="G46" s="5"/>
@@ -3029,7 +3290,9 @@
         <v>98</v>
       </c>
       <c r="I46" s="5"/>
-      <c r="J46" s="5"/>
+      <c r="J46" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="47" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A47" s="3" t="s">
@@ -3041,7 +3304,9 @@
       <c r="C47" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="D47" s="5"/>
+      <c r="D47" s="5" t="s">
+        <v>478</v>
+      </c>
       <c r="E47" s="5"/>
       <c r="F47" s="5"/>
       <c r="G47" s="5"/>
@@ -3049,7 +3314,9 @@
         <v>98</v>
       </c>
       <c r="I47" s="5"/>
-      <c r="J47" s="5"/>
+      <c r="J47" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="48" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="3" t="s">
@@ -3061,7 +3328,9 @@
       <c r="C48" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="D48" s="5"/>
+      <c r="D48" s="5" t="s">
+        <v>478</v>
+      </c>
       <c r="E48" s="5"/>
       <c r="F48" s="5"/>
       <c r="G48" s="5"/>
@@ -3069,7 +3338,9 @@
         <v>98</v>
       </c>
       <c r="I48" s="5"/>
-      <c r="J48" s="5"/>
+      <c r="J48" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="49" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A49" s="3" t="s">
@@ -3081,7 +3352,9 @@
       <c r="C49" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="D49" s="5"/>
+      <c r="D49" s="5" t="s">
+        <v>478</v>
+      </c>
       <c r="E49" s="5"/>
       <c r="F49" s="5"/>
       <c r="G49" s="5"/>
@@ -3089,7 +3362,9 @@
         <v>98</v>
       </c>
       <c r="I49" s="5"/>
-      <c r="J49" s="5"/>
+      <c r="J49" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="50" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A50" s="3" t="s">
@@ -3101,7 +3376,9 @@
       <c r="C50" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="D50" s="5"/>
+      <c r="D50" s="5" t="s">
+        <v>478</v>
+      </c>
       <c r="E50" s="5"/>
       <c r="F50" s="5"/>
       <c r="G50" s="5"/>
@@ -3109,7 +3386,9 @@
         <v>98</v>
       </c>
       <c r="I50" s="5"/>
-      <c r="J50" s="5"/>
+      <c r="J50" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="51" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="3" t="s">
@@ -3121,7 +3400,9 @@
       <c r="C51" s="5" t="s">
         <v>65</v>
       </c>
-      <c r="D51" s="5"/>
+      <c r="D51" s="5" t="s">
+        <v>478</v>
+      </c>
       <c r="E51" s="5"/>
       <c r="F51" s="5"/>
       <c r="G51" s="5"/>
@@ -3129,7 +3410,9 @@
         <v>98</v>
       </c>
       <c r="I51" s="5"/>
-      <c r="J51" s="5"/>
+      <c r="J51" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="52" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A52" s="3" t="s">
@@ -3149,7 +3432,9 @@
         <v>98</v>
       </c>
       <c r="I52" s="5"/>
-      <c r="J52" s="5"/>
+      <c r="J52" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="53" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="3" t="s">
@@ -3169,7 +3454,9 @@
         <v>98</v>
       </c>
       <c r="I53" s="5"/>
-      <c r="J53" s="5"/>
+      <c r="J53" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="54" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A54" s="3" t="s">
@@ -3189,7 +3476,9 @@
         <v>98</v>
       </c>
       <c r="I54" s="5"/>
-      <c r="J54" s="5"/>
+      <c r="J54" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="55" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="3" t="s">
@@ -3209,7 +3498,9 @@
         <v>98</v>
       </c>
       <c r="I55" s="5"/>
-      <c r="J55" s="5"/>
+      <c r="J55" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="56" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A56" s="3" t="s">
@@ -3229,7 +3520,9 @@
         <v>98</v>
       </c>
       <c r="I56" s="5"/>
-      <c r="J56" s="5"/>
+      <c r="J56" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="57" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="3" t="s">
@@ -3249,7 +3542,9 @@
         <v>98</v>
       </c>
       <c r="I57" s="5"/>
-      <c r="J57" s="5"/>
+      <c r="J57" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="58" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="3" t="s">
@@ -3269,7 +3564,9 @@
         <v>98</v>
       </c>
       <c r="I58" s="5"/>
-      <c r="J58" s="5"/>
+      <c r="J58" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="59" spans="1:10" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="3" t="s">
@@ -3289,7 +3586,9 @@
         <v>98</v>
       </c>
       <c r="I59" s="5"/>
-      <c r="J59" s="5"/>
+      <c r="J59" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="60" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A60" s="3" t="s">
@@ -3309,7 +3608,9 @@
         <v>98</v>
       </c>
       <c r="I60" s="5"/>
-      <c r="J60" s="5"/>
+      <c r="J60" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="61" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A61" s="3" t="s">
@@ -3331,7 +3632,9 @@
         <v>67</v>
       </c>
       <c r="I61" s="5"/>
-      <c r="J61" s="5"/>
+      <c r="J61" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="62" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A62" s="3" t="s">
@@ -3353,7 +3656,9 @@
         <v>103</v>
       </c>
       <c r="I62" s="5"/>
-      <c r="J62" s="5"/>
+      <c r="J62" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="63" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A63" s="3" t="s">
@@ -3375,7 +3680,9 @@
         <v>99</v>
       </c>
       <c r="I63" s="5"/>
-      <c r="J63" s="5"/>
+      <c r="J63" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="64" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A64" s="3" t="s">
@@ -3388,7 +3695,7 @@
         <v>68</v>
       </c>
       <c r="D64" s="5" t="s">
-        <v>271</v>
+        <v>272</v>
       </c>
       <c r="E64" s="5"/>
       <c r="F64" s="5"/>
@@ -3397,7 +3704,9 @@
         <v>99</v>
       </c>
       <c r="I64" s="5"/>
-      <c r="J64" s="5"/>
+      <c r="J64" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="65" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A65" s="3" t="s">
@@ -3419,7 +3728,9 @@
         <v>99</v>
       </c>
       <c r="I65" s="5"/>
-      <c r="J65" s="5"/>
+      <c r="J65" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="66" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A66" s="3" t="s">
@@ -3441,7 +3752,9 @@
         <v>99</v>
       </c>
       <c r="I66" s="5"/>
-      <c r="J66" s="5"/>
+      <c r="J66" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="67" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A67" s="3" t="s">
@@ -3463,7 +3776,9 @@
         <v>99</v>
       </c>
       <c r="I67" s="5"/>
-      <c r="J67" s="5"/>
+      <c r="J67" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="68" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A68" s="3" t="s">
@@ -3485,7 +3800,9 @@
         <v>99</v>
       </c>
       <c r="I68" s="5"/>
-      <c r="J68" s="5"/>
+      <c r="J68" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="69" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A69" s="3" t="s">
@@ -3507,7 +3824,9 @@
         <v>99</v>
       </c>
       <c r="I69" s="5"/>
-      <c r="J69" s="5"/>
+      <c r="J69" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="70" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A70" s="3" t="s">
@@ -3529,7 +3848,9 @@
         <v>99</v>
       </c>
       <c r="I70" s="5"/>
-      <c r="J70" s="5"/>
+      <c r="J70" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="71" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A71" s="3" t="s">
@@ -3551,7 +3872,9 @@
         <v>99</v>
       </c>
       <c r="I71" s="5"/>
-      <c r="J71" s="5"/>
+      <c r="J71" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="72" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A72" s="3" t="s">
@@ -3573,7 +3896,9 @@
         <v>99</v>
       </c>
       <c r="I72" s="5"/>
-      <c r="J72" s="5"/>
+      <c r="J72" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="73" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A73" s="3" t="s">
@@ -3595,7 +3920,9 @@
         <v>99</v>
       </c>
       <c r="I73" s="5"/>
-      <c r="J73" s="5"/>
+      <c r="J73" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="74" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A74" s="3" t="s">
@@ -3617,7 +3944,9 @@
         <v>99</v>
       </c>
       <c r="I74" s="5"/>
-      <c r="J74" s="5"/>
+      <c r="J74" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="75" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A75" s="3" t="s">
@@ -3639,7 +3968,9 @@
         <v>99</v>
       </c>
       <c r="I75" s="5"/>
-      <c r="J75" s="5"/>
+      <c r="J75" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="76" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A76" s="3" t="s">
@@ -3661,7 +3992,9 @@
         <v>99</v>
       </c>
       <c r="I76" s="5"/>
-      <c r="J76" s="5"/>
+      <c r="J76" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="77" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A77" s="3" t="s">
@@ -3683,7 +4016,9 @@
         <v>99</v>
       </c>
       <c r="I77" s="5"/>
-      <c r="J77" s="5"/>
+      <c r="J77" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="78" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A78" s="3" t="s">
@@ -3705,7 +4040,9 @@
         <v>99</v>
       </c>
       <c r="I78" s="5"/>
-      <c r="J78" s="5"/>
+      <c r="J78" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="79" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A79" s="3" t="s">
@@ -3727,7 +4064,9 @@
         <v>99</v>
       </c>
       <c r="I79" s="5"/>
-      <c r="J79" s="5"/>
+      <c r="J79" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="80" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A80" s="3" t="s">
@@ -3749,7 +4088,9 @@
         <v>99</v>
       </c>
       <c r="I80" s="5"/>
-      <c r="J80" s="5"/>
+      <c r="J80" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="81" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A81" s="3" t="s">
@@ -3771,7 +4112,9 @@
         <v>99</v>
       </c>
       <c r="I81" s="5"/>
-      <c r="J81" s="5"/>
+      <c r="J81" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="82" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A82" s="3" t="s">
@@ -3793,7 +4136,9 @@
         <v>99</v>
       </c>
       <c r="I82" s="5"/>
-      <c r="J82" s="5"/>
+      <c r="J82" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="83" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A83" s="3" t="s">
@@ -3811,9 +4156,13 @@
       <c r="E83" s="5"/>
       <c r="F83" s="5"/>
       <c r="G83" s="5"/>
-      <c r="H83" s="5"/>
+      <c r="H83" s="5" t="s">
+        <v>104</v>
+      </c>
       <c r="I83" s="5"/>
-      <c r="J83" s="5"/>
+      <c r="J83" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="84" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A84" s="3" t="s">
@@ -3831,9 +4180,13 @@
       <c r="E84" s="5"/>
       <c r="F84" s="5"/>
       <c r="G84" s="5"/>
-      <c r="H84" s="5"/>
+      <c r="H84" s="5" t="s">
+        <v>100</v>
+      </c>
       <c r="I84" s="5"/>
-      <c r="J84" s="5"/>
+      <c r="J84" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="85" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A85" s="3" t="s">
@@ -3851,9 +4204,13 @@
       <c r="E85" s="5"/>
       <c r="F85" s="5"/>
       <c r="G85" s="5"/>
-      <c r="H85" s="5"/>
+      <c r="H85" s="5" t="s">
+        <v>100</v>
+      </c>
       <c r="I85" s="5"/>
-      <c r="J85" s="5"/>
+      <c r="J85" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="86" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A86" s="3" t="s">
@@ -3871,9 +4228,13 @@
       <c r="E86" s="5"/>
       <c r="F86" s="5"/>
       <c r="G86" s="5"/>
-      <c r="H86" s="5"/>
+      <c r="H86" s="5" t="s">
+        <v>100</v>
+      </c>
       <c r="I86" s="5"/>
-      <c r="J86" s="5"/>
+      <c r="J86" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="87" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A87" s="3" t="s">
@@ -3891,9 +4252,13 @@
       <c r="E87" s="5"/>
       <c r="F87" s="5"/>
       <c r="G87" s="5"/>
-      <c r="H87" s="5"/>
+      <c r="H87" s="5" t="s">
+        <v>100</v>
+      </c>
       <c r="I87" s="5"/>
-      <c r="J87" s="5"/>
+      <c r="J87" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="88" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A88" s="3" t="s">
@@ -3911,9 +4276,13 @@
       <c r="E88" s="5"/>
       <c r="F88" s="5"/>
       <c r="G88" s="5"/>
-      <c r="H88" s="5"/>
+      <c r="H88" s="5" t="s">
+        <v>100</v>
+      </c>
       <c r="I88" s="5"/>
-      <c r="J88" s="5"/>
+      <c r="J88" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="89" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A89" s="3" t="s">
@@ -3931,9 +4300,13 @@
       <c r="E89" s="5"/>
       <c r="F89" s="5"/>
       <c r="G89" s="5"/>
-      <c r="H89" s="5"/>
+      <c r="H89" s="5" t="s">
+        <v>100</v>
+      </c>
       <c r="I89" s="5"/>
-      <c r="J89" s="5"/>
+      <c r="J89" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="90" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A90" s="3" t="s">
@@ -3951,9 +4324,13 @@
       <c r="E90" s="5"/>
       <c r="F90" s="5"/>
       <c r="G90" s="5"/>
-      <c r="H90" s="5"/>
+      <c r="H90" s="5" t="s">
+        <v>100</v>
+      </c>
       <c r="I90" s="5"/>
-      <c r="J90" s="5"/>
+      <c r="J90" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="91" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A91" s="3" t="s">
@@ -3971,9 +4348,13 @@
       <c r="E91" s="5"/>
       <c r="F91" s="5"/>
       <c r="G91" s="5"/>
-      <c r="H91" s="5"/>
+      <c r="H91" s="5" t="s">
+        <v>100</v>
+      </c>
       <c r="I91" s="5"/>
-      <c r="J91" s="5"/>
+      <c r="J91" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="92" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A92" s="3" t="s">
@@ -3991,9 +4372,13 @@
       <c r="E92" s="5"/>
       <c r="F92" s="5"/>
       <c r="G92" s="5"/>
-      <c r="H92" s="5"/>
+      <c r="H92" s="5" t="s">
+        <v>100</v>
+      </c>
       <c r="I92" s="5"/>
-      <c r="J92" s="5"/>
+      <c r="J92" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="93" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A93" s="3" t="s">
@@ -4011,9 +4396,13 @@
       <c r="E93" s="5"/>
       <c r="F93" s="5"/>
       <c r="G93" s="5"/>
-      <c r="H93" s="5"/>
+      <c r="H93" s="5" t="s">
+        <v>105</v>
+      </c>
       <c r="I93" s="5"/>
-      <c r="J93" s="5"/>
+      <c r="J93" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="94" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A94" s="3" t="s">
@@ -4031,9 +4420,13 @@
       <c r="E94" s="5"/>
       <c r="F94" s="5"/>
       <c r="G94" s="5"/>
-      <c r="H94" s="5"/>
+      <c r="H94" s="5" t="s">
+        <v>105</v>
+      </c>
       <c r="I94" s="5"/>
-      <c r="J94" s="5"/>
+      <c r="J94" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="95" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A95" s="3" t="s">
@@ -4051,9 +4444,13 @@
       <c r="E95" s="5"/>
       <c r="F95" s="5"/>
       <c r="G95" s="5"/>
-      <c r="H95" s="5"/>
+      <c r="H95" s="5" t="s">
+        <v>101</v>
+      </c>
       <c r="I95" s="5"/>
-      <c r="J95" s="5"/>
+      <c r="J95" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="96" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A96" s="3" t="s">
@@ -4071,9 +4468,13 @@
       <c r="E96" s="5"/>
       <c r="F96" s="5"/>
       <c r="G96" s="5"/>
-      <c r="H96" s="5"/>
+      <c r="H96" s="5" t="s">
+        <v>105</v>
+      </c>
       <c r="I96" s="5"/>
-      <c r="J96" s="5"/>
+      <c r="J96" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="97" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A97" s="3" t="s">
@@ -4091,9 +4492,13 @@
       <c r="E97" s="5"/>
       <c r="F97" s="5"/>
       <c r="G97" s="5"/>
-      <c r="H97" s="5"/>
+      <c r="H97" s="5" t="s">
+        <v>101</v>
+      </c>
       <c r="I97" s="5"/>
-      <c r="J97" s="5"/>
+      <c r="J97" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="98" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A98" s="3" t="s">
@@ -4111,9 +4516,13 @@
       <c r="E98" s="5"/>
       <c r="F98" s="5"/>
       <c r="G98" s="5"/>
-      <c r="H98" s="5"/>
+      <c r="H98" s="5" t="s">
+        <v>101</v>
+      </c>
       <c r="I98" s="5"/>
-      <c r="J98" s="5"/>
+      <c r="J98" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="99" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A99" s="3" t="s">
@@ -4131,9 +4540,13 @@
       <c r="E99" s="5"/>
       <c r="F99" s="5"/>
       <c r="G99" s="5"/>
-      <c r="H99" s="5"/>
+      <c r="H99" s="5" t="s">
+        <v>101</v>
+      </c>
       <c r="I99" s="5"/>
-      <c r="J99" s="5"/>
+      <c r="J99" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="100" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A100" s="3" t="s">
@@ -4151,9 +4564,13 @@
       <c r="E100" s="5"/>
       <c r="F100" s="5"/>
       <c r="G100" s="5"/>
-      <c r="H100" s="5"/>
+      <c r="H100" s="5" t="s">
+        <v>101</v>
+      </c>
       <c r="I100" s="5"/>
-      <c r="J100" s="5"/>
+      <c r="J100" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="101" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A101" s="3" t="s">
@@ -4171,9 +4588,13 @@
       <c r="E101" s="5"/>
       <c r="F101" s="5"/>
       <c r="G101" s="5"/>
-      <c r="H101" s="5"/>
+      <c r="H101" s="5" t="s">
+        <v>101</v>
+      </c>
       <c r="I101" s="5"/>
-      <c r="J101" s="5"/>
+      <c r="J101" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="102" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A102" s="3" t="s">
@@ -4191,9 +4612,13 @@
       <c r="E102" s="5"/>
       <c r="F102" s="5"/>
       <c r="G102" s="5"/>
-      <c r="H102" s="5"/>
+      <c r="H102" s="5" t="s">
+        <v>101</v>
+      </c>
       <c r="I102" s="5"/>
-      <c r="J102" s="5"/>
+      <c r="J102" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="103" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A103" s="3" t="s">
@@ -4211,9 +4636,13 @@
       <c r="E103" s="5"/>
       <c r="F103" s="5"/>
       <c r="G103" s="5"/>
-      <c r="H103" s="5"/>
+      <c r="H103" s="5" t="s">
+        <v>101</v>
+      </c>
       <c r="I103" s="5"/>
-      <c r="J103" s="5"/>
+      <c r="J103" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="104" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A104" s="3" t="s">
@@ -4231,9 +4660,13 @@
       <c r="E104" s="5"/>
       <c r="F104" s="5"/>
       <c r="G104" s="5"/>
-      <c r="H104" s="5"/>
+      <c r="H104" s="5" t="s">
+        <v>101</v>
+      </c>
       <c r="I104" s="5"/>
-      <c r="J104" s="5"/>
+      <c r="J104" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="105" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A105" s="3" t="s">
@@ -4251,9 +4684,13 @@
       <c r="E105" s="5"/>
       <c r="F105" s="5"/>
       <c r="G105" s="5"/>
-      <c r="H105" s="5"/>
+      <c r="H105" s="5" t="s">
+        <v>101</v>
+      </c>
       <c r="I105" s="5"/>
-      <c r="J105" s="5"/>
+      <c r="J105" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="106" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A106" s="3" t="s">
@@ -4265,13 +4702,19 @@
       <c r="C106" s="5" t="s">
         <v>77</v>
       </c>
-      <c r="D106" s="5"/>
+      <c r="D106" s="5" t="s">
+        <v>344</v>
+      </c>
       <c r="E106" s="5"/>
       <c r="F106" s="5"/>
       <c r="G106" s="5"/>
-      <c r="H106" s="5"/>
+      <c r="H106" s="5" t="s">
+        <v>101</v>
+      </c>
       <c r="I106" s="5"/>
-      <c r="J106" s="5"/>
+      <c r="J106" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="107" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A107" s="3" t="s">
@@ -4289,9 +4732,13 @@
       <c r="E107" s="5"/>
       <c r="F107" s="5"/>
       <c r="G107" s="5"/>
-      <c r="H107" s="5"/>
+      <c r="H107" s="5" t="s">
+        <v>101</v>
+      </c>
       <c r="I107" s="5"/>
-      <c r="J107" s="5"/>
+      <c r="J107" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="108" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A108" s="3" t="s">
@@ -4309,9 +4756,13 @@
       <c r="E108" s="5"/>
       <c r="F108" s="5"/>
       <c r="G108" s="5"/>
-      <c r="H108" s="5"/>
+      <c r="H108" s="5" t="s">
+        <v>105</v>
+      </c>
       <c r="I108" s="5"/>
-      <c r="J108" s="5"/>
+      <c r="J108" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="109" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A109" s="3" t="s">
@@ -4329,9 +4780,13 @@
       <c r="E109" s="5"/>
       <c r="F109" s="5"/>
       <c r="G109" s="5"/>
-      <c r="H109" s="5"/>
+      <c r="H109" s="5" t="s">
+        <v>101</v>
+      </c>
       <c r="I109" s="5"/>
-      <c r="J109" s="5"/>
+      <c r="J109" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="110" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A110" s="3" t="s">
@@ -4349,9 +4804,13 @@
       <c r="E110" s="5"/>
       <c r="F110" s="5"/>
       <c r="G110" s="5"/>
-      <c r="H110" s="5"/>
+      <c r="H110" s="5" t="s">
+        <v>101</v>
+      </c>
       <c r="I110" s="5"/>
-      <c r="J110" s="5"/>
+      <c r="J110" s="5" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="111" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A111" s="3" t="s">
@@ -4369,9 +4828,13 @@
       <c r="E111" s="5"/>
       <c r="F111" s="5"/>
       <c r="G111" s="5"/>
-      <c r="H111" s="5"/>
+      <c r="H111" s="5" t="s">
+        <v>101</v>
+      </c>
       <c r="I111" s="5"/>
-      <c r="J111" s="5"/>
+      <c r="J111" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="112" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A112" s="3" t="s">
@@ -4389,9 +4852,13 @@
       <c r="E112" s="5"/>
       <c r="F112" s="5"/>
       <c r="G112" s="5"/>
-      <c r="H112" s="5"/>
+      <c r="H112" s="5" t="s">
+        <v>101</v>
+      </c>
       <c r="I112" s="5"/>
-      <c r="J112" s="5"/>
+      <c r="J112" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="113" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A113" s="3" t="s">
@@ -4407,9 +4874,13 @@
       <c r="E113" s="5"/>
       <c r="F113" s="5"/>
       <c r="G113" s="5"/>
-      <c r="H113" s="5"/>
+      <c r="H113" s="5" t="s">
+        <v>105</v>
+      </c>
       <c r="I113" s="5"/>
-      <c r="J113" s="5"/>
+      <c r="J113" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="114" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A114" s="3" t="s">
@@ -4427,9 +4898,13 @@
       <c r="E114" s="5"/>
       <c r="F114" s="5"/>
       <c r="G114" s="5"/>
-      <c r="H114" s="5"/>
+      <c r="H114" s="5" t="s">
+        <v>508</v>
+      </c>
       <c r="I114" s="5"/>
-      <c r="J114" s="5"/>
+      <c r="J114" s="5" t="s">
+        <v>18</v>
+      </c>
     </row>
     <row r="115" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A115" s="3" t="s">
@@ -4447,9 +4922,13 @@
       <c r="E115" s="5"/>
       <c r="F115" s="5"/>
       <c r="G115" s="5"/>
-      <c r="H115" s="5"/>
+      <c r="H115" s="5" t="s">
+        <v>94</v>
+      </c>
       <c r="I115" s="5"/>
-      <c r="J115" s="5"/>
+      <c r="J115" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="116" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A116" s="3" t="s">
@@ -4465,9 +4944,13 @@
       <c r="E116" s="5"/>
       <c r="F116" s="5"/>
       <c r="G116" s="5"/>
-      <c r="H116" s="5"/>
+      <c r="H116" s="5" t="s">
+        <v>94</v>
+      </c>
       <c r="I116" s="5"/>
-      <c r="J116" s="5"/>
+      <c r="J116" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="117" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A117" s="3" t="s">
@@ -4485,9 +4968,13 @@
       <c r="E117" s="5"/>
       <c r="F117" s="5"/>
       <c r="G117" s="5"/>
-      <c r="H117" s="5"/>
+      <c r="H117" s="5" t="s">
+        <v>94</v>
+      </c>
       <c r="I117" s="5"/>
-      <c r="J117" s="5"/>
+      <c r="J117" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="118" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A118" s="3" t="s">
@@ -4503,9 +4990,13 @@
       <c r="E118" s="5"/>
       <c r="F118" s="5"/>
       <c r="G118" s="5"/>
-      <c r="H118" s="5"/>
+      <c r="H118" s="5" t="s">
+        <v>94</v>
+      </c>
       <c r="I118" s="5"/>
-      <c r="J118" s="5"/>
+      <c r="J118" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="119" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A119" s="3" t="s">
@@ -4521,9 +5012,13 @@
       <c r="E119" s="5"/>
       <c r="F119" s="5"/>
       <c r="G119" s="5"/>
-      <c r="H119" s="5"/>
+      <c r="H119" s="5" t="s">
+        <v>98</v>
+      </c>
       <c r="I119" s="5"/>
-      <c r="J119" s="5"/>
+      <c r="J119" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="120" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A120" s="3" t="s">
@@ -4539,9 +5034,13 @@
       <c r="E120" s="5"/>
       <c r="F120" s="5"/>
       <c r="G120" s="5"/>
-      <c r="H120" s="5"/>
+      <c r="H120" s="5" t="s">
+        <v>98</v>
+      </c>
       <c r="I120" s="5"/>
-      <c r="J120" s="5"/>
+      <c r="J120" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="121" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A121" s="3" t="s">
@@ -4553,13 +5052,19 @@
       <c r="C121" s="5" t="s">
         <v>62</v>
       </c>
-      <c r="D121" s="5"/>
+      <c r="D121" s="5" t="s">
+        <v>376</v>
+      </c>
       <c r="E121" s="5"/>
       <c r="F121" s="5"/>
       <c r="G121" s="5"/>
-      <c r="H121" s="5"/>
+      <c r="H121" s="5" t="s">
+        <v>98</v>
+      </c>
       <c r="I121" s="5"/>
-      <c r="J121" s="5"/>
+      <c r="J121" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="122" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A122" s="3" t="s">
@@ -4577,9 +5082,13 @@
       <c r="E122" s="5"/>
       <c r="F122" s="5"/>
       <c r="G122" s="5"/>
-      <c r="H122" s="5"/>
+      <c r="H122" s="5" t="s">
+        <v>98</v>
+      </c>
       <c r="I122" s="5"/>
-      <c r="J122" s="5"/>
+      <c r="J122" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="123" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A123" s="3" t="s">
@@ -4597,9 +5106,13 @@
       <c r="E123" s="5"/>
       <c r="F123" s="5"/>
       <c r="G123" s="5"/>
-      <c r="H123" s="5"/>
+      <c r="H123" s="5" t="s">
+        <v>98</v>
+      </c>
       <c r="I123" s="5"/>
-      <c r="J123" s="5"/>
+      <c r="J123" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="124" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A124" s="3" t="s">
@@ -4617,9 +5130,13 @@
       <c r="E124" s="5"/>
       <c r="F124" s="5"/>
       <c r="G124" s="5"/>
-      <c r="H124" s="5"/>
+      <c r="H124" s="5" t="s">
+        <v>98</v>
+      </c>
       <c r="I124" s="5"/>
-      <c r="J124" s="5"/>
+      <c r="J124" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="125" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A125" s="3" t="s">
@@ -4637,9 +5154,13 @@
       <c r="E125" s="5"/>
       <c r="F125" s="5"/>
       <c r="G125" s="5"/>
-      <c r="H125" s="5"/>
+      <c r="H125" s="5" t="s">
+        <v>98</v>
+      </c>
       <c r="I125" s="5"/>
-      <c r="J125" s="5"/>
+      <c r="J125" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="126" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A126" s="3" t="s">
@@ -4657,9 +5178,13 @@
       <c r="E126" s="5"/>
       <c r="F126" s="5"/>
       <c r="G126" s="5"/>
-      <c r="H126" s="5"/>
+      <c r="H126" s="5" t="s">
+        <v>98</v>
+      </c>
       <c r="I126" s="5"/>
-      <c r="J126" s="5"/>
+      <c r="J126" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="127" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A127" s="3" t="s">
@@ -4677,9 +5202,13 @@
       <c r="E127" s="5"/>
       <c r="F127" s="5"/>
       <c r="G127" s="5"/>
-      <c r="H127" s="5"/>
+      <c r="H127" s="5" t="s">
+        <v>98</v>
+      </c>
       <c r="I127" s="5"/>
-      <c r="J127" s="5"/>
+      <c r="J127" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="128" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A128" s="3" t="s">
@@ -4697,9 +5226,13 @@
       <c r="E128" s="5"/>
       <c r="F128" s="5"/>
       <c r="G128" s="5"/>
-      <c r="H128" s="5"/>
+      <c r="H128" s="5" t="s">
+        <v>98</v>
+      </c>
       <c r="I128" s="5"/>
-      <c r="J128" s="5"/>
+      <c r="J128" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="129" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A129" s="3" t="s">
@@ -4711,13 +5244,19 @@
       <c r="C129" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="D129" s="5"/>
+      <c r="D129" s="5" t="s">
+        <v>479</v>
+      </c>
       <c r="E129" s="5"/>
       <c r="F129" s="5"/>
       <c r="G129" s="5"/>
-      <c r="H129" s="5"/>
+      <c r="H129" s="5" t="s">
+        <v>94</v>
+      </c>
       <c r="I129" s="5"/>
-      <c r="J129" s="5"/>
+      <c r="J129" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="130" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A130" s="3" t="s">
@@ -4729,13 +5268,19 @@
       <c r="C130" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="D130" s="5"/>
+      <c r="D130" s="5" t="s">
+        <v>479</v>
+      </c>
       <c r="E130" s="5"/>
       <c r="F130" s="5"/>
       <c r="G130" s="5"/>
-      <c r="H130" s="5"/>
+      <c r="H130" s="5" t="s">
+        <v>94</v>
+      </c>
       <c r="I130" s="5"/>
-      <c r="J130" s="5"/>
+      <c r="J130" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="131" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A131" s="3" t="s">
@@ -4747,13 +5292,19 @@
       <c r="C131" s="5" t="s">
         <v>95</v>
       </c>
-      <c r="D131" s="5"/>
+      <c r="D131" s="5" t="s">
+        <v>479</v>
+      </c>
       <c r="E131" s="5"/>
       <c r="F131" s="5"/>
       <c r="G131" s="5"/>
-      <c r="H131" s="5"/>
+      <c r="H131" s="5" t="s">
+        <v>94</v>
+      </c>
       <c r="I131" s="5"/>
-      <c r="J131" s="5"/>
+      <c r="J131" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="132" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A132" s="3" t="s">
@@ -4769,245 +5320,413 @@
       <c r="E132" s="5"/>
       <c r="F132" s="5"/>
       <c r="G132" s="5"/>
-      <c r="H132" s="5"/>
+      <c r="H132" s="5" t="s">
+        <v>94</v>
+      </c>
       <c r="I132" s="5"/>
-      <c r="J132" s="5"/>
+      <c r="J132" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="133" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A133" s="3" t="s">
         <v>323</v>
       </c>
-      <c r="B133" s="5"/>
-      <c r="C133" s="5"/>
-      <c r="D133" s="5"/>
+      <c r="B133" s="5" t="s">
+        <v>458</v>
+      </c>
+      <c r="C133" s="5" t="s">
+        <v>400</v>
+      </c>
+      <c r="D133" s="5" t="s">
+        <v>280</v>
+      </c>
       <c r="E133" s="5"/>
       <c r="F133" s="5"/>
       <c r="G133" s="5"/>
-      <c r="H133" s="5"/>
+      <c r="H133" s="5" t="s">
+        <v>97</v>
+      </c>
       <c r="I133" s="5"/>
-      <c r="J133" s="5"/>
+      <c r="J133" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="134" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A134" s="3" t="s">
         <v>324</v>
       </c>
-      <c r="B134" s="5"/>
-      <c r="C134" s="5"/>
-      <c r="D134" s="5"/>
+      <c r="B134" s="5" t="s">
+        <v>459</v>
+      </c>
+      <c r="C134" s="5" t="s">
+        <v>400</v>
+      </c>
+      <c r="D134" s="5" t="s">
+        <v>280</v>
+      </c>
       <c r="E134" s="5"/>
       <c r="F134" s="5"/>
       <c r="G134" s="5"/>
-      <c r="H134" s="5"/>
+      <c r="H134" s="5" t="s">
+        <v>97</v>
+      </c>
       <c r="I134" s="5"/>
-      <c r="J134" s="5"/>
+      <c r="J134" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="135" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A135" s="3" t="s">
         <v>325</v>
       </c>
-      <c r="B135" s="5"/>
-      <c r="C135" s="5"/>
-      <c r="D135" s="5"/>
+      <c r="B135" s="5" t="s">
+        <v>460</v>
+      </c>
+      <c r="C135" s="5" t="s">
+        <v>400</v>
+      </c>
+      <c r="D135" s="5" t="s">
+        <v>280</v>
+      </c>
       <c r="E135" s="5"/>
       <c r="F135" s="5"/>
       <c r="G135" s="5"/>
-      <c r="H135" s="5"/>
+      <c r="H135" s="5" t="s">
+        <v>97</v>
+      </c>
       <c r="I135" s="5"/>
-      <c r="J135" s="5"/>
+      <c r="J135" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="136" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A136" s="3" t="s">
         <v>326</v>
       </c>
-      <c r="B136" s="5"/>
-      <c r="C136" s="5"/>
-      <c r="D136" s="5"/>
+      <c r="B136" s="5" t="s">
+        <v>461</v>
+      </c>
+      <c r="C136" s="5" t="s">
+        <v>400</v>
+      </c>
+      <c r="D136" s="5" t="s">
+        <v>280</v>
+      </c>
       <c r="E136" s="5"/>
       <c r="F136" s="5"/>
       <c r="G136" s="5"/>
-      <c r="H136" s="5"/>
+      <c r="H136" s="5" t="s">
+        <v>97</v>
+      </c>
       <c r="I136" s="5"/>
-      <c r="J136" s="5"/>
+      <c r="J136" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="137" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A137" s="3" t="s">
         <v>327</v>
       </c>
-      <c r="B137" s="5"/>
-      <c r="C137" s="5"/>
-      <c r="D137" s="5"/>
+      <c r="B137" s="5" t="s">
+        <v>462</v>
+      </c>
+      <c r="C137" s="5" t="s">
+        <v>400</v>
+      </c>
+      <c r="D137" s="5" t="s">
+        <v>280</v>
+      </c>
       <c r="E137" s="5"/>
       <c r="F137" s="5"/>
       <c r="G137" s="5"/>
-      <c r="H137" s="5"/>
+      <c r="H137" s="5" t="s">
+        <v>97</v>
+      </c>
       <c r="I137" s="5"/>
-      <c r="J137" s="5"/>
+      <c r="J137" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="138" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A138" s="3" t="s">
         <v>328</v>
       </c>
-      <c r="B138" s="5"/>
-      <c r="C138" s="5"/>
-      <c r="D138" s="5"/>
+      <c r="B138" s="5" t="s">
+        <v>463</v>
+      </c>
+      <c r="C138" s="5" t="s">
+        <v>473</v>
+      </c>
+      <c r="D138" s="5" t="s">
+        <v>280</v>
+      </c>
       <c r="E138" s="5"/>
       <c r="F138" s="5"/>
       <c r="G138" s="5"/>
-      <c r="H138" s="5"/>
+      <c r="H138" s="5" t="s">
+        <v>98</v>
+      </c>
       <c r="I138" s="5"/>
-      <c r="J138" s="5"/>
+      <c r="J138" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="139" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A139" s="3" t="s">
         <v>329</v>
       </c>
-      <c r="B139" s="5"/>
-      <c r="C139" s="5"/>
-      <c r="D139" s="5"/>
+      <c r="B139" s="5" t="s">
+        <v>464</v>
+      </c>
+      <c r="C139" s="5" t="s">
+        <v>473</v>
+      </c>
+      <c r="D139" s="5" t="s">
+        <v>280</v>
+      </c>
       <c r="E139" s="5"/>
       <c r="F139" s="5"/>
       <c r="G139" s="5"/>
-      <c r="H139" s="5"/>
+      <c r="H139" s="5" t="s">
+        <v>98</v>
+      </c>
       <c r="I139" s="5"/>
-      <c r="J139" s="5"/>
+      <c r="J139" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="140" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A140" s="3" t="s">
         <v>330</v>
       </c>
-      <c r="B140" s="5"/>
-      <c r="C140" s="5"/>
-      <c r="D140" s="5"/>
+      <c r="B140" s="5" t="s">
+        <v>465</v>
+      </c>
+      <c r="C140" s="5" t="s">
+        <v>473</v>
+      </c>
+      <c r="D140" s="5" t="s">
+        <v>280</v>
+      </c>
       <c r="E140" s="5"/>
       <c r="F140" s="5"/>
       <c r="G140" s="5"/>
-      <c r="H140" s="5"/>
+      <c r="H140" s="5" t="s">
+        <v>98</v>
+      </c>
       <c r="I140" s="5"/>
-      <c r="J140" s="5"/>
+      <c r="J140" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="141" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A141" s="3" t="s">
         <v>331</v>
       </c>
-      <c r="B141" s="5"/>
-      <c r="C141" s="5"/>
-      <c r="D141" s="5"/>
+      <c r="B141" s="5" t="s">
+        <v>466</v>
+      </c>
+      <c r="C141" s="5" t="s">
+        <v>473</v>
+      </c>
+      <c r="D141" s="5" t="s">
+        <v>280</v>
+      </c>
       <c r="E141" s="5"/>
       <c r="F141" s="5"/>
       <c r="G141" s="5"/>
-      <c r="H141" s="5"/>
+      <c r="H141" s="5" t="s">
+        <v>98</v>
+      </c>
       <c r="I141" s="5"/>
-      <c r="J141" s="5"/>
+      <c r="J141" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="142" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A142" s="3" t="s">
         <v>332</v>
       </c>
-      <c r="B142" s="5"/>
-      <c r="C142" s="5"/>
-      <c r="D142" s="5"/>
+      <c r="B142" s="5" t="s">
+        <v>467</v>
+      </c>
+      <c r="C142" s="5" t="s">
+        <v>473</v>
+      </c>
+      <c r="D142" s="5" t="s">
+        <v>280</v>
+      </c>
       <c r="E142" s="5"/>
       <c r="F142" s="5"/>
       <c r="G142" s="5"/>
-      <c r="H142" s="5"/>
+      <c r="H142" s="5" t="s">
+        <v>102</v>
+      </c>
       <c r="I142" s="5"/>
-      <c r="J142" s="5"/>
+      <c r="J142" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="143" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A143" s="3" t="s">
         <v>333</v>
       </c>
-      <c r="B143" s="5"/>
-      <c r="C143" s="5"/>
-      <c r="D143" s="5"/>
+      <c r="B143" s="5" t="s">
+        <v>468</v>
+      </c>
+      <c r="C143" s="5" t="s">
+        <v>471</v>
+      </c>
+      <c r="D143" s="5" t="s">
+        <v>280</v>
+      </c>
       <c r="E143" s="5"/>
       <c r="F143" s="5"/>
       <c r="G143" s="5"/>
-      <c r="H143" s="5"/>
+      <c r="H143" s="5" t="s">
+        <v>98</v>
+      </c>
       <c r="I143" s="5"/>
-      <c r="J143" s="5"/>
+      <c r="J143" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="144" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A144" s="3" t="s">
         <v>334</v>
       </c>
-      <c r="B144" s="5"/>
-      <c r="C144" s="5"/>
-      <c r="D144" s="5"/>
+      <c r="B144" s="5" t="s">
+        <v>469</v>
+      </c>
+      <c r="C144" s="5" t="s">
+        <v>471</v>
+      </c>
+      <c r="D144" s="5" t="s">
+        <v>480</v>
+      </c>
       <c r="E144" s="5"/>
       <c r="F144" s="5"/>
       <c r="G144" s="5"/>
-      <c r="H144" s="5"/>
+      <c r="H144" s="5" t="s">
+        <v>508</v>
+      </c>
       <c r="I144" s="5"/>
-      <c r="J144" s="5"/>
+      <c r="J144" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="145" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A145" s="3" t="s">
         <v>335</v>
       </c>
-      <c r="B145" s="5"/>
-      <c r="C145" s="5"/>
+      <c r="B145" s="5" t="s">
+        <v>470</v>
+      </c>
+      <c r="C145" s="5" t="s">
+        <v>471</v>
+      </c>
       <c r="D145" s="5"/>
       <c r="E145" s="5"/>
       <c r="F145" s="5"/>
       <c r="G145" s="5"/>
-      <c r="H145" s="5"/>
+      <c r="H145" s="5" t="s">
+        <v>508</v>
+      </c>
       <c r="I145" s="5"/>
-      <c r="J145" s="5"/>
+      <c r="J145" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="146" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A146" s="3" t="s">
         <v>336</v>
       </c>
-      <c r="B146" s="5"/>
-      <c r="C146" s="5"/>
-      <c r="D146" s="5"/>
+      <c r="B146" s="5" t="s">
+        <v>93</v>
+      </c>
+      <c r="C146" s="5" t="s">
+        <v>471</v>
+      </c>
+      <c r="D146" s="5" t="s">
+        <v>280</v>
+      </c>
       <c r="E146" s="5"/>
       <c r="F146" s="5"/>
       <c r="G146" s="5"/>
-      <c r="H146" s="5"/>
+      <c r="H146" s="5" t="s">
+        <v>93</v>
+      </c>
       <c r="I146" s="5"/>
-      <c r="J146" s="5"/>
+      <c r="J146" s="5" t="s">
+        <v>444</v>
+      </c>
     </row>
     <row r="147" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A147" s="3" t="s">
         <v>337</v>
       </c>
-      <c r="B147" s="5"/>
-      <c r="C147" s="5"/>
-      <c r="D147" s="5"/>
+      <c r="B147" s="5" t="s">
+        <v>481</v>
+      </c>
+      <c r="C147" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="D147" s="5" t="s">
+        <v>507</v>
+      </c>
       <c r="E147" s="5"/>
       <c r="F147" s="5"/>
       <c r="G147" s="5"/>
-      <c r="H147" s="5"/>
+      <c r="H147" s="5" t="s">
+        <v>508</v>
+      </c>
       <c r="I147" s="5"/>
-      <c r="J147" s="5"/>
+      <c r="J147" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="148" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A148" s="3" t="s">
         <v>338</v>
       </c>
-      <c r="B148" s="5"/>
-      <c r="C148" s="5"/>
-      <c r="D148" s="5"/>
+      <c r="B148" s="5" t="s">
+        <v>482</v>
+      </c>
+      <c r="C148" s="5" t="s">
+        <v>506</v>
+      </c>
+      <c r="D148" s="5" t="s">
+        <v>507</v>
+      </c>
       <c r="E148" s="5"/>
       <c r="F148" s="5"/>
       <c r="G148" s="5"/>
-      <c r="H148" s="5"/>
+      <c r="H148" s="5" t="s">
+        <v>508</v>
+      </c>
       <c r="I148" s="5"/>
-      <c r="J148" s="5"/>
+      <c r="J148" s="5" t="s">
+        <v>14</v>
+      </c>
     </row>
     <row r="149" spans="1:10" x14ac:dyDescent="0.3">
       <c r="A149" s="3" t="s">
         <v>339</v>
       </c>
-      <c r="B149" s="5"/>
-      <c r="C149" s="5"/>
+      <c r="B149" s="5" t="s">
+        <v>509</v>
+      </c>
+      <c r="C149" s="5" t="s">
+        <v>471</v>
+      </c>
       <c r="D149" s="5"/>
       <c r="E149" s="5"/>
       <c r="F149" s="5"/>
       <c r="G149" s="5"/>
-      <c r="H149" s="5"/>
+      <c r="H149" s="5" t="s">
+        <v>107</v>
+      </c>
       <c r="I149" s="5"/>
       <c r="J149" s="5"/>
     </row>
@@ -5015,15 +5734,353 @@
       <c r="A150" s="3" t="s">
         <v>340</v>
       </c>
-      <c r="B150" s="5"/>
-      <c r="C150" s="5"/>
+      <c r="B150" s="5" t="s">
+        <v>510</v>
+      </c>
+      <c r="C150" s="5" t="s">
+        <v>471</v>
+      </c>
       <c r="D150" s="5"/>
       <c r="E150" s="5"/>
       <c r="F150" s="5"/>
       <c r="G150" s="5"/>
-      <c r="H150" s="5"/>
+      <c r="H150" s="5" t="s">
+        <v>99</v>
+      </c>
       <c r="I150" s="5"/>
       <c r="J150" s="5"/>
+    </row>
+    <row r="151" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A151" s="3" t="s">
+        <v>483</v>
+      </c>
+      <c r="B151" s="5" t="s">
+        <v>511</v>
+      </c>
+      <c r="C151" s="5" t="s">
+        <v>471</v>
+      </c>
+      <c r="D151" s="5"/>
+      <c r="E151" s="5"/>
+      <c r="F151" s="5"/>
+      <c r="G151" s="5"/>
+      <c r="H151" s="5" t="s">
+        <v>99</v>
+      </c>
+      <c r="I151" s="5"/>
+      <c r="J151" s="5"/>
+    </row>
+    <row r="152" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A152" s="3" t="s">
+        <v>484</v>
+      </c>
+      <c r="B152" s="5" t="s">
+        <v>512</v>
+      </c>
+      <c r="C152" s="5" t="s">
+        <v>471</v>
+      </c>
+      <c r="D152" s="5"/>
+      <c r="E152" s="5"/>
+      <c r="F152" s="5"/>
+      <c r="G152" s="5"/>
+      <c r="H152" s="5"/>
+      <c r="I152" s="5"/>
+      <c r="J152" s="5"/>
+    </row>
+    <row r="153" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A153" s="3" t="s">
+        <v>485</v>
+      </c>
+      <c r="B153" s="5"/>
+      <c r="C153" s="5"/>
+      <c r="D153" s="5"/>
+      <c r="E153" s="5"/>
+      <c r="F153" s="5"/>
+      <c r="G153" s="5"/>
+      <c r="H153" s="5"/>
+      <c r="I153" s="5"/>
+      <c r="J153" s="5"/>
+    </row>
+    <row r="154" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A154" s="3" t="s">
+        <v>486</v>
+      </c>
+      <c r="B154" s="5"/>
+      <c r="C154" s="5"/>
+      <c r="D154" s="5"/>
+      <c r="E154" s="5"/>
+      <c r="F154" s="5"/>
+      <c r="G154" s="5"/>
+      <c r="H154" s="5"/>
+      <c r="I154" s="5"/>
+      <c r="J154" s="5"/>
+    </row>
+    <row r="155" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A155" s="3" t="s">
+        <v>487</v>
+      </c>
+      <c r="B155" s="5"/>
+      <c r="C155" s="5"/>
+      <c r="D155" s="5"/>
+      <c r="E155" s="5"/>
+      <c r="F155" s="5"/>
+      <c r="G155" s="5"/>
+      <c r="H155" s="5"/>
+      <c r="I155" s="5"/>
+      <c r="J155" s="5"/>
+    </row>
+    <row r="156" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A156" s="3" t="s">
+        <v>488</v>
+      </c>
+      <c r="B156" s="5"/>
+      <c r="C156" s="5"/>
+      <c r="D156" s="5"/>
+      <c r="E156" s="5"/>
+      <c r="F156" s="5"/>
+      <c r="G156" s="5"/>
+      <c r="H156" s="5"/>
+      <c r="I156" s="5"/>
+      <c r="J156" s="5"/>
+    </row>
+    <row r="157" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A157" s="3" t="s">
+        <v>489</v>
+      </c>
+      <c r="B157" s="5"/>
+      <c r="C157" s="5"/>
+      <c r="D157" s="5"/>
+      <c r="E157" s="5"/>
+      <c r="F157" s="5"/>
+      <c r="G157" s="5"/>
+      <c r="H157" s="5"/>
+      <c r="I157" s="5"/>
+      <c r="J157" s="5"/>
+    </row>
+    <row r="158" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A158" s="3" t="s">
+        <v>490</v>
+      </c>
+      <c r="B158" s="5"/>
+      <c r="C158" s="5"/>
+      <c r="D158" s="5"/>
+      <c r="E158" s="5"/>
+      <c r="F158" s="5"/>
+      <c r="G158" s="5"/>
+      <c r="H158" s="5"/>
+      <c r="I158" s="5"/>
+      <c r="J158" s="5"/>
+    </row>
+    <row r="159" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A159" s="3" t="s">
+        <v>491</v>
+      </c>
+      <c r="B159" s="5"/>
+      <c r="C159" s="5"/>
+      <c r="D159" s="5"/>
+      <c r="E159" s="5"/>
+      <c r="F159" s="5"/>
+      <c r="G159" s="5"/>
+      <c r="H159" s="5"/>
+      <c r="I159" s="5"/>
+      <c r="J159" s="5"/>
+    </row>
+    <row r="160" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A160" s="3" t="s">
+        <v>492</v>
+      </c>
+      <c r="B160" s="5"/>
+      <c r="C160" s="5"/>
+      <c r="D160" s="5"/>
+      <c r="E160" s="5"/>
+      <c r="F160" s="5"/>
+      <c r="G160" s="5"/>
+      <c r="H160" s="5"/>
+      <c r="I160" s="5"/>
+      <c r="J160" s="5"/>
+    </row>
+    <row r="161" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A161" s="3" t="s">
+        <v>493</v>
+      </c>
+      <c r="B161" s="5"/>
+      <c r="C161" s="5"/>
+      <c r="D161" s="5"/>
+      <c r="E161" s="5"/>
+      <c r="F161" s="5"/>
+      <c r="G161" s="5"/>
+      <c r="H161" s="5"/>
+      <c r="I161" s="5"/>
+      <c r="J161" s="5"/>
+    </row>
+    <row r="162" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A162" s="3" t="s">
+        <v>494</v>
+      </c>
+      <c r="B162" s="5"/>
+      <c r="C162" s="5"/>
+      <c r="D162" s="5"/>
+      <c r="E162" s="5"/>
+      <c r="F162" s="5"/>
+      <c r="G162" s="5"/>
+      <c r="H162" s="5"/>
+      <c r="I162" s="5"/>
+      <c r="J162" s="5"/>
+    </row>
+    <row r="163" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A163" s="3" t="s">
+        <v>495</v>
+      </c>
+      <c r="B163" s="5"/>
+      <c r="C163" s="5"/>
+      <c r="D163" s="5"/>
+      <c r="E163" s="5"/>
+      <c r="F163" s="5"/>
+      <c r="G163" s="5"/>
+      <c r="H163" s="5"/>
+      <c r="I163" s="5"/>
+      <c r="J163" s="5"/>
+    </row>
+    <row r="164" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A164" s="3" t="s">
+        <v>496</v>
+      </c>
+      <c r="B164" s="5"/>
+      <c r="C164" s="5"/>
+      <c r="D164" s="5"/>
+      <c r="E164" s="5"/>
+      <c r="F164" s="5"/>
+      <c r="G164" s="5"/>
+      <c r="H164" s="5"/>
+      <c r="I164" s="5"/>
+      <c r="J164" s="5"/>
+    </row>
+    <row r="165" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A165" s="3" t="s">
+        <v>497</v>
+      </c>
+      <c r="B165" s="5"/>
+      <c r="C165" s="5"/>
+      <c r="D165" s="5"/>
+      <c r="E165" s="5"/>
+      <c r="F165" s="5"/>
+      <c r="G165" s="5"/>
+      <c r="H165" s="5"/>
+      <c r="I165" s="5"/>
+      <c r="J165" s="5"/>
+    </row>
+    <row r="166" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A166" s="3" t="s">
+        <v>498</v>
+      </c>
+      <c r="B166" s="5"/>
+      <c r="C166" s="5"/>
+      <c r="D166" s="5"/>
+      <c r="E166" s="5"/>
+      <c r="F166" s="5"/>
+      <c r="G166" s="5"/>
+      <c r="H166" s="5"/>
+      <c r="I166" s="5"/>
+      <c r="J166" s="5"/>
+    </row>
+    <row r="167" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A167" s="3" t="s">
+        <v>499</v>
+      </c>
+      <c r="B167" s="5"/>
+      <c r="C167" s="5"/>
+      <c r="D167" s="5"/>
+      <c r="E167" s="5"/>
+      <c r="F167" s="5"/>
+      <c r="G167" s="5"/>
+      <c r="H167" s="5"/>
+      <c r="I167" s="5"/>
+      <c r="J167" s="5"/>
+    </row>
+    <row r="168" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A168" s="3" t="s">
+        <v>500</v>
+      </c>
+      <c r="B168" s="5"/>
+      <c r="C168" s="5"/>
+      <c r="D168" s="5"/>
+      <c r="E168" s="5"/>
+      <c r="F168" s="5"/>
+      <c r="G168" s="5"/>
+      <c r="H168" s="5"/>
+      <c r="I168" s="5"/>
+      <c r="J168" s="5"/>
+    </row>
+    <row r="169" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A169" s="3" t="s">
+        <v>501</v>
+      </c>
+      <c r="B169" s="5"/>
+      <c r="C169" s="5"/>
+      <c r="D169" s="5"/>
+      <c r="E169" s="5"/>
+      <c r="F169" s="5"/>
+      <c r="G169" s="5"/>
+      <c r="H169" s="5"/>
+      <c r="I169" s="5"/>
+      <c r="J169" s="5"/>
+    </row>
+    <row r="170" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A170" s="3" t="s">
+        <v>502</v>
+      </c>
+      <c r="B170" s="5"/>
+      <c r="C170" s="5"/>
+      <c r="D170" s="5"/>
+      <c r="E170" s="5"/>
+      <c r="F170" s="5"/>
+      <c r="G170" s="5"/>
+      <c r="H170" s="5"/>
+      <c r="I170" s="5"/>
+      <c r="J170" s="5"/>
+    </row>
+    <row r="171" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A171" s="3" t="s">
+        <v>503</v>
+      </c>
+      <c r="B171" s="5"/>
+      <c r="C171" s="5"/>
+      <c r="D171" s="5"/>
+      <c r="E171" s="5"/>
+      <c r="F171" s="5"/>
+      <c r="G171" s="5"/>
+      <c r="H171" s="5"/>
+      <c r="I171" s="5"/>
+      <c r="J171" s="5"/>
+    </row>
+    <row r="172" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A172" s="3" t="s">
+        <v>504</v>
+      </c>
+      <c r="B172" s="5"/>
+      <c r="C172" s="5"/>
+      <c r="D172" s="5"/>
+      <c r="E172" s="5"/>
+      <c r="F172" s="5"/>
+      <c r="G172" s="5"/>
+      <c r="H172" s="5"/>
+      <c r="I172" s="5"/>
+      <c r="J172" s="5"/>
+    </row>
+    <row r="173" spans="1:10" x14ac:dyDescent="0.3">
+      <c r="A173" s="3" t="s">
+        <v>505</v>
+      </c>
+      <c r="B173" s="5"/>
+      <c r="C173" s="5"/>
+      <c r="D173" s="5"/>
+      <c r="E173" s="5"/>
+      <c r="F173" s="5"/>
+      <c r="G173" s="5"/>
+      <c r="H173" s="5"/>
+      <c r="I173" s="5"/>
+      <c r="J173" s="5"/>
     </row>
   </sheetData>
   <mergeCells count="8">
@@ -5095,57 +6152,57 @@
   <sheetPr>
     <tabColor rgb="FF375623"/>
   </sheetPr>
-  <dimension ref="A1:AF30"/>
+  <dimension ref="A1:AL30"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="29" width="23.109375" customWidth="1"/>
     <col min="30" max="38" width="17.88671875" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:32" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A1" s="19" t="s">
+    <row r="1" spans="1:38" ht="31.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A1" s="24" t="s">
         <v>20</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="14"/>
-      <c r="G1" s="14"/>
-      <c r="H1" s="14"/>
-    </row>
-    <row r="2" spans="1:32" ht="18" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A2" s="15" t="s">
+      <c r="B1" s="19"/>
+      <c r="C1" s="19"/>
+      <c r="D1" s="19"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="19"/>
+      <c r="G1" s="19"/>
+      <c r="H1" s="19"/>
+    </row>
+    <row r="2" spans="1:38" ht="18" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A2" s="20" t="s">
         <v>21</v>
       </c>
-      <c r="B2" s="14"/>
-      <c r="C2" s="14"/>
-      <c r="D2" s="14"/>
-      <c r="E2" s="14"/>
-      <c r="F2" s="14"/>
-      <c r="G2" s="14"/>
-      <c r="H2" s="14"/>
-    </row>
-    <row r="3" spans="1:32" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A3" s="20" t="s">
+      <c r="B2" s="19"/>
+      <c r="C2" s="19"/>
+      <c r="D2" s="19"/>
+      <c r="E2" s="19"/>
+      <c r="F2" s="19"/>
+      <c r="G2" s="19"/>
+      <c r="H2" s="19"/>
+    </row>
+    <row r="3" spans="1:38" ht="25.95" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A3" s="12" t="s">
         <v>66</v>
       </c>
-      <c r="B3" s="20" t="s">
+      <c r="B3" s="12" t="s">
         <v>58</v>
       </c>
-      <c r="C3" s="20" t="s">
+      <c r="C3" s="12" t="s">
         <v>59</v>
       </c>
-      <c r="D3" s="20" t="s">
+      <c r="D3" s="12" t="s">
         <v>63</v>
       </c>
-      <c r="E3" s="20" t="s">
+      <c r="E3" s="12" t="s">
         <v>64</v>
       </c>
-      <c r="F3" s="20" t="s">
+      <c r="F3" s="12" t="s">
         <v>61</v>
       </c>
-      <c r="G3" s="20" t="s">
+      <c r="G3" s="12" t="s">
         <v>95</v>
       </c>
       <c r="H3" s="11" t="s">
@@ -5166,9 +6223,7 @@
       <c r="M3" s="11" t="s">
         <v>69</v>
       </c>
-      <c r="N3" s="11" t="s">
-        <v>400</v>
-      </c>
+      <c r="N3" s="11"/>
       <c r="O3" s="11" t="s">
         <v>401</v>
       </c>
@@ -5223,589 +6278,720 @@
       <c r="AF3" s="11" t="s">
         <v>377</v>
       </c>
-    </row>
-    <row r="4" spans="1:32" s="22" customFormat="1" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A4" s="21" t="s">
+      <c r="AG3" s="11" t="s">
+        <v>400</v>
+      </c>
+      <c r="AH3" s="11" t="s">
+        <v>471</v>
+      </c>
+      <c r="AI3" s="11" t="s">
+        <v>473</v>
+      </c>
+      <c r="AJ3" s="11" t="s">
+        <v>513</v>
+      </c>
+      <c r="AK3" s="11" t="s">
+        <v>512</v>
+      </c>
+      <c r="AL3" s="11" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="4" spans="1:38" s="8" customFormat="1" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="13" t="s">
         <v>109</v>
       </c>
-      <c r="B4" s="21" t="s">
+      <c r="B4" s="13" t="s">
         <v>114</v>
       </c>
-      <c r="C4" s="21" t="s">
+      <c r="C4" s="13" t="s">
         <v>119</v>
       </c>
-      <c r="D4" s="21" t="s">
+      <c r="D4" s="13" t="s">
         <v>124</v>
       </c>
-      <c r="E4" s="21" t="s">
+      <c r="E4" s="13" t="s">
         <v>128</v>
       </c>
-      <c r="F4" s="21" t="s">
+      <c r="F4" s="13" t="s">
         <v>380</v>
       </c>
-      <c r="G4" s="21" t="s">
+      <c r="G4" s="13" t="s">
         <v>384</v>
       </c>
-      <c r="H4" s="22" t="s">
+      <c r="H4" s="8" t="s">
         <v>402</v>
       </c>
-      <c r="I4" s="22" t="s">
+      <c r="I4" s="8" t="s">
         <v>402</v>
       </c>
-      <c r="J4" s="22" t="s">
+      <c r="J4" s="8" t="s">
         <v>402</v>
       </c>
-      <c r="K4" s="22" t="s">
+      <c r="K4" s="8" t="s">
         <v>402</v>
       </c>
-      <c r="L4" s="22" t="s">
+      <c r="L4" s="8" t="s">
         <v>402</v>
       </c>
-      <c r="M4" s="22" t="s">
+      <c r="M4" s="8" t="s">
         <v>402</v>
       </c>
-      <c r="N4" s="22" t="s">
+      <c r="O4" s="8" t="s">
         <v>402</v>
       </c>
-      <c r="O4" s="22" t="s">
+      <c r="P4" s="8" t="s">
         <v>402</v>
       </c>
-      <c r="P4" s="22" t="s">
+      <c r="Q4" s="8" t="s">
         <v>402</v>
       </c>
-      <c r="Q4" s="22" t="s">
+      <c r="R4" s="8" t="s">
         <v>402</v>
       </c>
-      <c r="R4" s="22" t="s">
+      <c r="S4" s="8" t="s">
         <v>402</v>
       </c>
-      <c r="S4" s="22" t="s">
+      <c r="T4" s="8" t="s">
         <v>402</v>
       </c>
-      <c r="T4" s="22" t="s">
+      <c r="U4" s="8" t="s">
         <v>402</v>
       </c>
-      <c r="U4" s="22" t="s">
+      <c r="V4" s="8" t="s">
         <v>402</v>
       </c>
-      <c r="V4" s="22" t="s">
+      <c r="W4" s="8" t="s">
         <v>402</v>
       </c>
-      <c r="W4" s="22" t="s">
+      <c r="X4" s="8" t="s">
         <v>402</v>
       </c>
-      <c r="X4" s="22" t="s">
+      <c r="Y4" s="8" t="s">
         <v>402</v>
       </c>
-      <c r="Y4" s="22" t="s">
+      <c r="Z4" s="8" t="s">
         <v>402</v>
       </c>
-      <c r="Z4" s="22" t="s">
+      <c r="AA4" s="8" t="s">
         <v>402</v>
       </c>
-      <c r="AA4" s="22" t="s">
+      <c r="AB4" s="8" t="s">
         <v>402</v>
       </c>
-      <c r="AB4" s="22" t="s">
+      <c r="AC4" s="8" t="s">
         <v>402</v>
       </c>
-      <c r="AC4" s="22" t="s">
+      <c r="AD4" s="8" t="s">
         <v>402</v>
       </c>
-      <c r="AD4" s="22" t="s">
+      <c r="AE4" s="8" t="s">
         <v>402</v>
       </c>
-      <c r="AE4" s="22" t="s">
+      <c r="AF4" s="8" t="s">
         <v>402</v>
       </c>
-      <c r="AF4" s="22" t="s">
+      <c r="AG4" s="8" t="s">
         <v>402</v>
       </c>
-    </row>
-    <row r="5" spans="1:32" s="24" customFormat="1" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A5" s="23" t="s">
+      <c r="AH4" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="AI4" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="AJ4" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="AK4" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="AL4" s="8" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="5" spans="1:38" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A5" s="14" t="s">
         <v>110</v>
       </c>
-      <c r="B5" s="23" t="s">
+      <c r="B5" s="14" t="s">
         <v>115</v>
       </c>
-      <c r="C5" s="23" t="s">
+      <c r="C5" s="14" t="s">
         <v>117</v>
       </c>
-      <c r="D5" s="23" t="s">
+      <c r="D5" s="14" t="s">
         <v>125</v>
       </c>
-      <c r="E5" s="23" t="s">
+      <c r="E5" s="14" t="s">
         <v>129</v>
       </c>
-      <c r="F5" s="23" t="s">
+      <c r="F5" s="14" t="s">
         <v>381</v>
       </c>
-      <c r="G5" s="23" t="s">
+      <c r="G5" s="14" t="s">
         <v>385</v>
       </c>
-      <c r="H5" s="23" t="s">
+      <c r="H5" s="14" t="s">
         <v>403</v>
       </c>
-      <c r="I5" s="23" t="s">
+      <c r="I5" s="14" t="s">
         <v>407</v>
       </c>
-      <c r="J5" s="23" t="s">
+      <c r="J5" s="14" t="s">
         <v>409</v>
       </c>
-      <c r="K5" s="23" t="s">
+      <c r="K5" s="14" t="s">
+        <v>446</v>
+      </c>
+      <c r="L5" s="14" t="s">
+        <v>413</v>
+      </c>
+      <c r="M5" s="14" t="s">
+        <v>416</v>
+      </c>
+      <c r="N5" s="14"/>
+      <c r="O5" s="14" t="s">
+        <v>445</v>
+      </c>
+      <c r="P5" s="14" t="s">
+        <v>418</v>
+      </c>
+      <c r="Q5" s="14" t="s">
+        <v>422</v>
+      </c>
+      <c r="R5" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="S5" s="14" t="s">
+        <v>423</v>
+      </c>
+      <c r="T5" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="U5" s="14" t="s">
+        <v>426</v>
+      </c>
+      <c r="V5" s="14" t="s">
+        <v>128</v>
+      </c>
+      <c r="W5" s="14" t="s">
+        <v>428</v>
+      </c>
+      <c r="X5" s="14" t="s">
+        <v>432</v>
+      </c>
+      <c r="Y5" s="14" t="s">
+        <v>433</v>
+      </c>
+      <c r="Z5" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="AA5" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="AB5" s="14" t="s">
+        <v>435</v>
+      </c>
+      <c r="AC5" s="14" t="s">
+        <v>436</v>
+      </c>
+      <c r="AD5" s="14" t="s">
+        <v>431</v>
+      </c>
+      <c r="AE5" s="14" t="s">
+        <v>440</v>
+      </c>
+      <c r="AF5" s="14" t="s">
+        <v>414</v>
+      </c>
+      <c r="AG5" s="14" t="s">
+        <v>414</v>
+      </c>
+      <c r="AH5" s="14" t="s">
+        <v>449</v>
+      </c>
+      <c r="AI5" s="14" t="s">
+        <v>474</v>
+      </c>
+      <c r="AJ5" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="AK5" s="14" t="s">
+        <v>473</v>
+      </c>
+      <c r="AL5" s="14" t="s">
         <v>412</v>
       </c>
-      <c r="L5" s="23" t="s">
+    </row>
+    <row r="6" spans="1:38" s="8" customFormat="1" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A6" s="13" t="s">
+        <v>111</v>
+      </c>
+      <c r="B6" s="13" t="s">
+        <v>116</v>
+      </c>
+      <c r="C6" s="13" t="s">
+        <v>120</v>
+      </c>
+      <c r="D6" s="13" t="s">
+        <v>115</v>
+      </c>
+      <c r="E6" s="13" t="s">
+        <v>130</v>
+      </c>
+      <c r="F6" s="13" t="s">
+        <v>382</v>
+      </c>
+      <c r="G6" s="13" t="s">
+        <v>386</v>
+      </c>
+      <c r="H6" s="8" t="s">
+        <v>404</v>
+      </c>
+      <c r="I6" s="8" t="s">
+        <v>403</v>
+      </c>
+      <c r="J6" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="K6" s="8" t="s">
+        <v>447</v>
+      </c>
+      <c r="L6" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="M6" s="8" t="s">
+        <v>417</v>
+      </c>
+      <c r="O6" s="13" t="s">
+        <v>448</v>
+      </c>
+      <c r="P6" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="Q6" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="R6" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="S6" s="8" t="s">
+        <v>424</v>
+      </c>
+      <c r="T6" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="U6" s="8" t="s">
+        <v>427</v>
+      </c>
+      <c r="V6" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="W6" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="X6" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="Y6" s="8" t="s">
+        <v>426</v>
+      </c>
+      <c r="Z6" s="8" t="s">
+        <v>477</v>
+      </c>
+      <c r="AA6" s="8" t="s">
+        <v>412</v>
+      </c>
+      <c r="AB6" s="8" t="s">
+        <v>426</v>
+      </c>
+      <c r="AC6" s="8" t="s">
+        <v>437</v>
+      </c>
+      <c r="AD6" s="8" t="s">
+        <v>438</v>
+      </c>
+      <c r="AE6" s="8" t="s">
+        <v>441</v>
+      </c>
+      <c r="AF6" s="8" t="s">
+        <v>412</v>
+      </c>
+      <c r="AG6" s="8" t="s">
+        <v>412</v>
+      </c>
+      <c r="AH6" s="8" t="s">
+        <v>472</v>
+      </c>
+      <c r="AI6" s="8" t="s">
+        <v>475</v>
+      </c>
+      <c r="AJ6" s="8" t="s">
+        <v>514</v>
+      </c>
+      <c r="AK6" s="8" t="s">
+        <v>118</v>
+      </c>
+      <c r="AL6" s="8" t="s">
+        <v>414</v>
+      </c>
+    </row>
+    <row r="7" spans="1:38" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A7" s="14" t="s">
+        <v>112</v>
+      </c>
+      <c r="B7" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="C7" s="14" t="s">
+        <v>121</v>
+      </c>
+      <c r="D7" s="14" t="s">
+        <v>126</v>
+      </c>
+      <c r="E7" s="14" t="s">
+        <v>131</v>
+      </c>
+      <c r="F7" s="14" t="s">
+        <v>383</v>
+      </c>
+      <c r="G7" s="14" t="s">
+        <v>387</v>
+      </c>
+      <c r="H7" s="14" t="s">
+        <v>381</v>
+      </c>
+      <c r="I7" s="14" t="s">
+        <v>408</v>
+      </c>
+      <c r="J7" s="14" t="s">
+        <v>125</v>
+      </c>
+      <c r="K7" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="L7" s="14" t="s">
+        <v>118</v>
+      </c>
+      <c r="M7" s="14" t="s">
+        <v>411</v>
+      </c>
+      <c r="N7" s="14"/>
+      <c r="O7" t="s">
+        <v>450</v>
+      </c>
+      <c r="P7" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="Q7" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="R7" s="14" t="s">
+        <v>411</v>
+      </c>
+      <c r="S7" s="14" t="s">
+        <v>425</v>
+      </c>
+      <c r="T7" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="U7" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="V7" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="W7" s="14" t="s">
+        <v>429</v>
+      </c>
+      <c r="X7" s="14" t="s">
+        <v>431</v>
+      </c>
+      <c r="Y7" s="14" t="s">
+        <v>417</v>
+      </c>
+      <c r="AA7" s="14" t="s">
+        <v>434</v>
+      </c>
+      <c r="AB7" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="AD7" s="14" t="s">
+        <v>412</v>
+      </c>
+      <c r="AE7" s="14" t="s">
+        <v>442</v>
+      </c>
+      <c r="AG7" s="14" t="s">
+        <v>452</v>
+      </c>
+      <c r="AH7" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="AI7" s="14" t="s">
+        <v>476</v>
+      </c>
+      <c r="AJ7" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="AK7" s="14" t="s">
+        <v>514</v>
+      </c>
+      <c r="AL7" s="14" t="s">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="8" spans="1:38" s="8" customFormat="1" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A8" s="13" t="s">
+        <v>113</v>
+      </c>
+      <c r="B8" s="13" t="s">
+        <v>118</v>
+      </c>
+      <c r="C8" s="13" t="s">
+        <v>122</v>
+      </c>
+      <c r="D8" s="13" t="s">
+        <v>127</v>
+      </c>
+      <c r="E8" s="13" t="s">
+        <v>132</v>
+      </c>
+      <c r="F8" s="8" t="s">
+        <v>402</v>
+      </c>
+      <c r="G8" s="13" t="s">
+        <v>388</v>
+      </c>
+      <c r="H8" s="8" t="s">
+        <v>405</v>
+      </c>
+      <c r="I8" s="8" t="s">
+        <v>365</v>
+      </c>
+      <c r="J8" s="8" t="s">
+        <v>410</v>
+      </c>
+      <c r="K8" s="8" t="s">
+        <v>412</v>
+      </c>
+      <c r="L8" s="8" t="s">
+        <v>414</v>
+      </c>
+      <c r="M8" s="8" t="s">
+        <v>134</v>
+      </c>
+      <c r="O8" s="8" t="s">
+        <v>451</v>
+      </c>
+      <c r="P8" s="8" t="s">
+        <v>420</v>
+      </c>
+      <c r="Q8" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="R8" s="8" t="s">
+        <v>123</v>
+      </c>
+      <c r="U8" s="8" t="s">
+        <v>124</v>
+      </c>
+      <c r="W8" s="8" t="s">
+        <v>430</v>
+      </c>
+      <c r="X8" s="8" t="s">
+        <v>412</v>
+      </c>
+      <c r="AA8" s="8" t="s">
+        <v>416</v>
+      </c>
+      <c r="AB8" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="AD8" s="8" t="s">
+        <v>439</v>
+      </c>
+      <c r="AE8" s="8" t="s">
+        <v>117</v>
+      </c>
+      <c r="AG8" s="13" t="s">
+        <v>453</v>
+      </c>
+      <c r="AI8" s="8" t="s">
+        <v>381</v>
+      </c>
+      <c r="AK8" s="8" t="s">
+        <v>515</v>
+      </c>
+    </row>
+    <row r="9" spans="1:38" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A9" s="15" t="s">
+        <v>402</v>
+      </c>
+      <c r="B9" s="15" t="s">
+        <v>402</v>
+      </c>
+      <c r="C9" s="14" t="s">
+        <v>123</v>
+      </c>
+      <c r="D9" s="15" t="s">
+        <v>402</v>
+      </c>
+      <c r="E9" s="14" t="s">
+        <v>133</v>
+      </c>
+      <c r="G9" s="14" t="s">
+        <v>389</v>
+      </c>
+      <c r="H9" s="14" t="s">
+        <v>406</v>
+      </c>
+      <c r="J9" s="14" t="s">
+        <v>127</v>
+      </c>
+      <c r="L9" s="14" t="s">
         <v>415</v>
       </c>
-      <c r="M5" s="23" t="s">
+      <c r="M9" s="14" t="s">
         <v>418</v>
       </c>
-      <c r="N5" s="23" t="s">
+      <c r="O9" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="R9" s="14" t="s">
+        <v>414</v>
+      </c>
+      <c r="W9" s="14" t="s">
+        <v>431</v>
+      </c>
+      <c r="X9" s="14" t="s">
+        <v>426</v>
+      </c>
+      <c r="AA9" s="14" t="s">
+        <v>124</v>
+      </c>
+      <c r="AE9" s="14" t="s">
+        <v>443</v>
+      </c>
+      <c r="AG9" s="14" t="s">
+        <v>454</v>
+      </c>
+      <c r="AI9" s="14" t="s">
+        <v>449</v>
+      </c>
+    </row>
+    <row r="10" spans="1:38" s="8" customFormat="1" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A10" s="16"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="16" t="s">
+        <v>402</v>
+      </c>
+      <c r="D10" s="16"/>
+      <c r="E10" s="13" t="s">
+        <v>134</v>
+      </c>
+      <c r="G10" s="13" t="s">
+        <v>390</v>
+      </c>
+      <c r="H10" s="8" t="s">
+        <v>361</v>
+      </c>
+      <c r="J10" s="8" t="s">
+        <v>411</v>
+      </c>
+      <c r="M10" s="8" t="s">
+        <v>419</v>
+      </c>
+      <c r="O10" s="8" t="s">
+        <v>421</v>
+      </c>
+      <c r="R10" s="8" t="s">
         <v>412</v>
       </c>
-      <c r="O5" s="23" t="s">
+      <c r="W10" s="8" t="s">
         <v>412</v>
       </c>
-      <c r="P5" s="23" t="s">
+      <c r="X10" s="8" t="s">
+        <v>416</v>
+      </c>
+      <c r="AG10" s="13" t="s">
+        <v>455</v>
+      </c>
+      <c r="AI10" s="8" t="s">
+        <v>472</v>
+      </c>
+    </row>
+    <row r="11" spans="1:38" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A11" s="15"/>
+      <c r="B11" s="15"/>
+      <c r="C11" s="15"/>
+      <c r="D11" s="15"/>
+      <c r="E11" s="14" t="s">
+        <v>117</v>
+      </c>
+      <c r="G11" t="s">
+        <v>402</v>
+      </c>
+      <c r="M11" s="14" t="s">
         <v>420</v>
       </c>
-      <c r="Q5" s="23" t="s">
-        <v>425</v>
-      </c>
-      <c r="R5" s="23" t="s">
-        <v>125</v>
-      </c>
-      <c r="S5" s="23" t="s">
-        <v>426</v>
-      </c>
-      <c r="T5" s="23" t="s">
-        <v>128</v>
-      </c>
-      <c r="U5" s="23" t="s">
-        <v>429</v>
-      </c>
-      <c r="V5" s="23" t="s">
-        <v>128</v>
-      </c>
-      <c r="W5" s="23" t="s">
-        <v>431</v>
-      </c>
-      <c r="X5" s="23" t="s">
-        <v>435</v>
-      </c>
-      <c r="Y5" s="23" t="s">
-        <v>436</v>
-      </c>
-      <c r="AA5" s="23" t="s">
-        <v>123</v>
-      </c>
-      <c r="AB5" s="23" t="s">
-        <v>438</v>
-      </c>
-      <c r="AC5" s="23" t="s">
-        <v>439</v>
-      </c>
-      <c r="AD5" s="23" t="s">
-        <v>434</v>
-      </c>
-      <c r="AE5" s="23" t="s">
-        <v>443</v>
-      </c>
-      <c r="AF5" s="23" t="s">
-        <v>416</v>
-      </c>
-    </row>
-    <row r="6" spans="1:32" s="22" customFormat="1" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A6" s="21" t="s">
-        <v>111</v>
-      </c>
-      <c r="B6" s="21" t="s">
-        <v>116</v>
-      </c>
-      <c r="C6" s="21" t="s">
-        <v>120</v>
-      </c>
-      <c r="D6" s="21" t="s">
-        <v>115</v>
-      </c>
-      <c r="E6" s="21" t="s">
-        <v>130</v>
-      </c>
-      <c r="F6" s="21" t="s">
-        <v>382</v>
-      </c>
-      <c r="G6" s="21" t="s">
-        <v>386</v>
-      </c>
-      <c r="H6" s="22" t="s">
-        <v>404</v>
-      </c>
-      <c r="I6" s="22" t="s">
-        <v>403</v>
-      </c>
-      <c r="J6" s="22" t="s">
+      <c r="R11" s="14" t="s">
         <v>117</v>
       </c>
-      <c r="K6" s="22" t="s">
-        <v>413</v>
-      </c>
-      <c r="L6" s="22" t="s">
+      <c r="W11" s="14" t="s">
         <v>117</v>
       </c>
-      <c r="M6" s="22" t="s">
-        <v>419</v>
-      </c>
-      <c r="N6" s="22" t="s">
-        <v>423</v>
-      </c>
-      <c r="O6" s="22" t="s">
-        <v>423</v>
-      </c>
-      <c r="P6" s="22" t="s">
-        <v>134</v>
-      </c>
-      <c r="Q6" s="22" t="s">
-        <v>123</v>
-      </c>
-      <c r="R6" s="22" t="s">
-        <v>124</v>
-      </c>
-      <c r="S6" s="22" t="s">
-        <v>427</v>
-      </c>
-      <c r="T6" s="22" t="s">
-        <v>124</v>
-      </c>
-      <c r="U6" s="22" t="s">
-        <v>430</v>
-      </c>
-      <c r="V6" s="22" t="s">
-        <v>124</v>
-      </c>
-      <c r="W6" s="22" t="s">
-        <v>123</v>
-      </c>
-      <c r="X6" s="22" t="s">
-        <v>123</v>
-      </c>
-      <c r="Y6" s="22" t="s">
-        <v>429</v>
-      </c>
-      <c r="AA6" s="22" t="s">
-        <v>414</v>
-      </c>
-      <c r="AB6" s="22" t="s">
-        <v>429</v>
-      </c>
-      <c r="AC6" s="22" t="s">
-        <v>440</v>
-      </c>
-      <c r="AD6" s="22" t="s">
-        <v>441</v>
-      </c>
-      <c r="AE6" s="22" t="s">
-        <v>444</v>
-      </c>
-      <c r="AF6" s="22" t="s">
-        <v>414</v>
-      </c>
-    </row>
-    <row r="7" spans="1:32" s="24" customFormat="1" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A7" s="23" t="s">
-        <v>112</v>
-      </c>
-      <c r="B7" s="23" t="s">
+      <c r="X11" s="14" t="s">
         <v>117</v>
       </c>
-      <c r="C7" s="23" t="s">
-        <v>121</v>
-      </c>
-      <c r="D7" s="23" t="s">
-        <v>126</v>
-      </c>
-      <c r="E7" s="23" t="s">
-        <v>131</v>
-      </c>
-      <c r="F7" s="23" t="s">
-        <v>383</v>
-      </c>
-      <c r="G7" s="23" t="s">
-        <v>387</v>
-      </c>
-      <c r="H7" s="23" t="s">
-        <v>381</v>
-      </c>
-      <c r="I7" s="23" t="s">
-        <v>408</v>
-      </c>
-      <c r="J7" s="23" t="s">
-        <v>125</v>
-      </c>
-      <c r="K7" s="23" t="s">
+      <c r="AG11" s="14" t="s">
+        <v>450</v>
+      </c>
+      <c r="AI11" s="14" t="s">
         <v>117</v>
       </c>
-      <c r="L7" s="23" t="s">
-        <v>118</v>
-      </c>
-      <c r="M7" s="23" t="s">
-        <v>411</v>
-      </c>
-      <c r="N7" s="23" t="s">
-        <v>117</v>
-      </c>
-      <c r="O7" s="23" t="s">
-        <v>117</v>
-      </c>
-      <c r="P7" s="23" t="s">
-        <v>124</v>
-      </c>
-      <c r="Q7" s="23" t="s">
-        <v>124</v>
-      </c>
-      <c r="R7" s="23" t="s">
-        <v>411</v>
-      </c>
-      <c r="S7" s="23" t="s">
-        <v>428</v>
-      </c>
-      <c r="T7" s="23" t="s">
-        <v>117</v>
-      </c>
-      <c r="U7" s="23" t="s">
-        <v>117</v>
-      </c>
-      <c r="V7" s="23" t="s">
-        <v>117</v>
-      </c>
-      <c r="W7" s="23" t="s">
-        <v>432</v>
-      </c>
-      <c r="X7" s="23" t="s">
-        <v>434</v>
-      </c>
-      <c r="Y7" s="23" t="s">
-        <v>419</v>
-      </c>
-      <c r="AA7" s="23" t="s">
-        <v>437</v>
-      </c>
-      <c r="AB7" s="23" t="s">
-        <v>123</v>
-      </c>
-      <c r="AD7" s="23" t="s">
-        <v>414</v>
-      </c>
-      <c r="AE7" s="23" t="s">
-        <v>445</v>
-      </c>
-    </row>
-    <row r="8" spans="1:32" s="22" customFormat="1" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A8" s="21" t="s">
-        <v>113</v>
-      </c>
-      <c r="B8" s="21" t="s">
-        <v>118</v>
-      </c>
-      <c r="C8" s="21" t="s">
-        <v>122</v>
-      </c>
-      <c r="D8" s="21" t="s">
-        <v>127</v>
-      </c>
-      <c r="E8" s="21" t="s">
-        <v>132</v>
-      </c>
-      <c r="F8" s="22" t="s">
+    </row>
+    <row r="12" spans="1:38" s="8" customFormat="1" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A12" s="16"/>
+      <c r="B12" s="16"/>
+      <c r="C12" s="16"/>
+      <c r="D12" s="16"/>
+      <c r="E12" s="13" t="s">
+        <v>135</v>
+      </c>
+      <c r="AG12" s="13" t="s">
+        <v>451</v>
+      </c>
+    </row>
+    <row r="13" spans="1:38" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A13" s="15"/>
+      <c r="B13" s="15"/>
+      <c r="C13" s="15"/>
+      <c r="D13" s="15"/>
+      <c r="E13" s="15" t="s">
         <v>402</v>
       </c>
-      <c r="G8" s="21" t="s">
-        <v>388</v>
-      </c>
-      <c r="H8" s="22" t="s">
-        <v>405</v>
-      </c>
-      <c r="I8" s="22" t="s">
-        <v>365</v>
-      </c>
-      <c r="J8" s="22" t="s">
-        <v>410</v>
-      </c>
-      <c r="K8" s="22" t="s">
-        <v>414</v>
-      </c>
-      <c r="L8" s="22" t="s">
-        <v>416</v>
-      </c>
-      <c r="M8" s="22" t="s">
-        <v>134</v>
-      </c>
-      <c r="N8" s="22" t="s">
-        <v>424</v>
-      </c>
-      <c r="O8" s="22" t="s">
-        <v>424</v>
-      </c>
-      <c r="P8" s="22" t="s">
-        <v>422</v>
-      </c>
-      <c r="Q8" s="22" t="s">
-        <v>117</v>
-      </c>
-      <c r="R8" s="22" t="s">
-        <v>123</v>
-      </c>
-      <c r="U8" s="22" t="s">
-        <v>124</v>
-      </c>
-      <c r="W8" s="22" t="s">
-        <v>433</v>
-      </c>
-      <c r="X8" s="22" t="s">
-        <v>414</v>
-      </c>
-      <c r="AA8" s="22" t="s">
-        <v>418</v>
-      </c>
-      <c r="AB8" s="22" t="s">
-        <v>117</v>
-      </c>
-      <c r="AD8" s="22" t="s">
-        <v>442</v>
-      </c>
-      <c r="AE8" s="22" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="9" spans="1:32" s="24" customFormat="1" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A9" s="25" t="s">
-        <v>402</v>
-      </c>
-      <c r="B9" s="25" t="s">
-        <v>402</v>
-      </c>
-      <c r="C9" s="23" t="s">
-        <v>123</v>
-      </c>
-      <c r="D9" s="25" t="s">
-        <v>402</v>
-      </c>
-      <c r="E9" s="23" t="s">
-        <v>133</v>
-      </c>
-      <c r="G9" s="23" t="s">
-        <v>389</v>
-      </c>
-      <c r="H9" s="23" t="s">
-        <v>406</v>
-      </c>
-      <c r="J9" s="23" t="s">
-        <v>127</v>
-      </c>
-      <c r="L9" s="23" t="s">
-        <v>417</v>
-      </c>
-      <c r="M9" s="23" t="s">
-        <v>420</v>
-      </c>
-      <c r="R9" s="23" t="s">
-        <v>416</v>
-      </c>
-      <c r="W9" s="23" t="s">
-        <v>434</v>
-      </c>
-      <c r="X9" s="23" t="s">
-        <v>429</v>
-      </c>
-      <c r="AE9" s="23" t="s">
-        <v>446</v>
-      </c>
-    </row>
-    <row r="10" spans="1:32" s="22" customFormat="1" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A10" s="26"/>
-      <c r="B10" s="26"/>
-      <c r="C10" s="26" t="s">
-        <v>402</v>
-      </c>
-      <c r="D10" s="26"/>
-      <c r="E10" s="21" t="s">
-        <v>134</v>
-      </c>
-      <c r="G10" s="21" t="s">
-        <v>390</v>
-      </c>
-      <c r="H10" s="22" t="s">
-        <v>361</v>
-      </c>
-      <c r="J10" s="22" t="s">
-        <v>411</v>
-      </c>
-      <c r="M10" s="22" t="s">
-        <v>421</v>
-      </c>
-      <c r="R10" s="22" t="s">
-        <v>414</v>
-      </c>
-      <c r="W10" s="22" t="s">
-        <v>414</v>
-      </c>
-      <c r="X10" s="22" t="s">
-        <v>418</v>
-      </c>
-    </row>
-    <row r="11" spans="1:32" s="24" customFormat="1" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A11" s="25"/>
-      <c r="B11" s="25"/>
-      <c r="C11" s="25"/>
-      <c r="D11" s="25"/>
-      <c r="E11" s="23" t="s">
-        <v>117</v>
-      </c>
-      <c r="G11" s="24" t="s">
-        <v>402</v>
-      </c>
-      <c r="M11" s="23" t="s">
-        <v>422</v>
-      </c>
-      <c r="R11" s="23" t="s">
-        <v>117</v>
-      </c>
-      <c r="W11" s="23" t="s">
-        <v>117</v>
-      </c>
-      <c r="X11" s="23" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="12" spans="1:32" s="22" customFormat="1" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A12" s="26"/>
-      <c r="B12" s="26"/>
-      <c r="C12" s="26"/>
-      <c r="D12" s="26"/>
-      <c r="E12" s="21" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="13" spans="1:32" s="24" customFormat="1" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A13" s="25"/>
-      <c r="B13" s="25"/>
-      <c r="C13" s="25"/>
-      <c r="D13" s="25"/>
-      <c r="E13" s="25" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="14" spans="1:32" s="22" customFormat="1" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="A14" s="26"/>
-      <c r="C14" s="26"/>
-      <c r="E14" s="26"/>
-    </row>
-    <row r="15" spans="1:32" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AG13" s="14" t="s">
+        <v>456</v>
+      </c>
+    </row>
+    <row r="14" spans="1:38" s="8" customFormat="1" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="A14" s="16"/>
+      <c r="C14" s="16"/>
+      <c r="E14" s="16"/>
+      <c r="AG14" s="13" t="s">
+        <v>457</v>
+      </c>
+    </row>
+    <row r="15" spans="1:38" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A15" s="7"/>
       <c r="E15" s="7"/>
-    </row>
-    <row r="16" spans="1:32" s="8" customFormat="1" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="AG15" s="14" t="s">
+        <v>117</v>
+      </c>
+    </row>
+    <row r="16" spans="1:38" s="8" customFormat="1" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="9"/>
     </row>
     <row r="17" spans="1:1" ht="16.05" customHeight="1" x14ac:dyDescent="0.3">
@@ -5823,13 +7009,14 @@
     <mergeCell ref="A2:H2"/>
     <mergeCell ref="A1:H1"/>
   </mergeCells>
+  <phoneticPr fontId="5" type="noConversion"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7417494D-5B4C-4190-AFD8-9808A78CEDC0}">
-  <dimension ref="B2:D35"/>
+  <dimension ref="B2:D38"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="26.88671875" customWidth="1"/>
@@ -5969,11 +7156,17 @@
       <c r="B19" s="10" t="s">
         <v>73</v>
       </c>
+      <c r="D19" t="s">
+        <v>508</v>
+      </c>
     </row>
     <row r="20" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B20" s="10" t="s">
         <v>74</v>
       </c>
+      <c r="D20" t="s">
+        <v>107</v>
+      </c>
     </row>
     <row r="21" spans="2:4" x14ac:dyDescent="0.3">
       <c r="B21" s="10" t="s">
@@ -6031,23 +7224,38 @@
       </c>
     </row>
     <row r="32" spans="2:4" x14ac:dyDescent="0.3">
-      <c r="B32" t="s">
+      <c r="B32" s="10" t="s">
         <v>96</v>
       </c>
     </row>
     <row r="33" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B33" t="s">
+      <c r="B33" s="10" t="s">
         <v>236</v>
       </c>
     </row>
     <row r="34" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B34" t="s">
+      <c r="B34" s="10" t="s">
         <v>253</v>
       </c>
     </row>
     <row r="35" spans="2:2" x14ac:dyDescent="0.3">
-      <c r="B35" t="s">
+      <c r="B35" s="10" t="s">
         <v>377</v>
+      </c>
+    </row>
+    <row r="36" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B36" s="10" t="s">
+        <v>471</v>
+      </c>
+    </row>
+    <row r="37" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B37" s="10" t="s">
+        <v>473</v>
+      </c>
+    </row>
+    <row r="38" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B38" s="10" t="s">
+        <v>506</v>
       </c>
     </row>
   </sheetData>

</xml_diff>